<commit_message>
filtered out trial 34 because a stimulus presentation mistake was made during this trial
also, added natcan 2025 data to excel file
</commit_message>
<xml_diff>
--- a/data/raw/2025/data_summer_2025.xlsx
+++ b/data/raw/2025/data_summer_2025.xlsx
@@ -1,21 +1,24 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10713"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10720"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://lunduniversityo365-my.sharepoint.com/personal/an4718sc_lu_se/Documents/PhD/projects/dorsal_snapshot_discrimination_project/analysis/data/raw/2025/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1" documentId="8_{BAD0E982-56D3-0E41-B109-60B516BAC403}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3E9F6D92-FE07-954F-A1B8-F0C0E4998D2B}"/>
+  <xr:revisionPtr revIDLastSave="563" documentId="8_{BAD0E982-56D3-0E41-B109-60B516BAC403}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5F871857-CC79-8647-A291-636AC4A09480}"/>
   <bookViews>
-    <workbookView xWindow="12520" yWindow="2040" windowWidth="28040" windowHeight="17440" activeTab="2" xr2:uid="{0F60F085-ABCE-EA48-9AAF-DAFB43BA76C4}"/>
+    <workbookView xWindow="4240" yWindow="2020" windowWidth="28040" windowHeight="17440" activeTab="2" xr2:uid="{0F60F085-ABCE-EA48-9AAF-DAFB43BA76C4}"/>
   </bookViews>
   <sheets>
     <sheet name="170725" sheetId="1" r:id="rId1"/>
     <sheet name="180725" sheetId="2" r:id="rId2"/>
     <sheet name="190725_ctrl" sheetId="3" r:id="rId3"/>
+    <sheet name="300725_natcan" sheetId="4" r:id="rId4"/>
+    <sheet name="310725natcan" sheetId="5" r:id="rId5"/>
+    <sheet name="010825natcan" sheetId="6" r:id="rId6"/>
   </sheets>
   <calcPr calcId="181029"/>
   <extLst>
@@ -38,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="423" uniqueCount="111">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="904" uniqueCount="139">
   <si>
     <t>individual</t>
   </si>
@@ -371,16 +374,107 @@
   </si>
   <si>
     <t>0,0,0,0,0,1</t>
+  </si>
+  <si>
+    <t>18L</t>
+  </si>
+  <si>
+    <t>19R</t>
+  </si>
+  <si>
+    <t>71L</t>
+  </si>
+  <si>
+    <t>72R</t>
+  </si>
+  <si>
+    <t>73L</t>
+  </si>
+  <si>
+    <t>74R</t>
+  </si>
+  <si>
+    <t>75L</t>
+  </si>
+  <si>
+    <t>76R</t>
+  </si>
+  <si>
+    <t>1,0,0,1,0</t>
+  </si>
+  <si>
+    <t>0,1,0,0,1,0,0</t>
+  </si>
+  <si>
+    <t>0,0,0,0,0,0,0,0,0</t>
+  </si>
+  <si>
+    <t>0,0,1,0,0,1</t>
+  </si>
+  <si>
+    <t>1,0,1,0,1</t>
+  </si>
+  <si>
+    <t>0,0,0,0,1,1</t>
+  </si>
+  <si>
+    <t>1,0,0,0,1</t>
+  </si>
+  <si>
+    <t>0,0,1,0,0,0</t>
+  </si>
+  <si>
+    <t>0,1,0,0,1</t>
+  </si>
+  <si>
+    <t>0,0,1,0,1</t>
+  </si>
+  <si>
+    <t>0,0,0,0,0,0</t>
+  </si>
+  <si>
+    <t>1 0</t>
+  </si>
+  <si>
+    <t>1,0,0,0,0,0</t>
+  </si>
+  <si>
+    <t>0,0,0,0,0,0,0,1</t>
+  </si>
+  <si>
+    <t>0,1,0,0</t>
+  </si>
+  <si>
+    <t>0,0,0,0,1,0</t>
+  </si>
+  <si>
+    <t>1,0,0,0,0,0,0</t>
+  </si>
+  <si>
+    <t>0,0,0,0,0,1,0</t>
+  </si>
+  <si>
+    <t>0,1,0,0,0,0,1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  </t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FF000000"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -412,9 +506,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -430,6 +525,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -2333,4 +2432,2405 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3367D427-091C-6946-8749-30AA4ADE2482}">
+  <dimension ref="A1:BY12"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetData>
+    <row r="1" spans="1:77" x14ac:dyDescent="0.2">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" t="s">
+        <v>9</v>
+      </c>
+      <c r="K1" t="s">
+        <v>10</v>
+      </c>
+      <c r="L1" t="s">
+        <v>11</v>
+      </c>
+      <c r="M1" t="s">
+        <v>12</v>
+      </c>
+      <c r="N1" t="s">
+        <v>13</v>
+      </c>
+      <c r="O1" t="s">
+        <v>14</v>
+      </c>
+      <c r="P1" t="s">
+        <v>15</v>
+      </c>
+      <c r="Q1" t="s">
+        <v>16</v>
+      </c>
+      <c r="R1" t="s">
+        <v>17</v>
+      </c>
+      <c r="S1" t="s">
+        <v>111</v>
+      </c>
+      <c r="T1" t="s">
+        <v>112</v>
+      </c>
+      <c r="U1" t="s">
+        <v>20</v>
+      </c>
+      <c r="V1" t="s">
+        <v>21</v>
+      </c>
+      <c r="W1" t="s">
+        <v>22</v>
+      </c>
+      <c r="X1" t="s">
+        <v>23</v>
+      </c>
+      <c r="Y1" t="s">
+        <v>24</v>
+      </c>
+      <c r="Z1" t="s">
+        <v>25</v>
+      </c>
+      <c r="AA1" t="s">
+        <v>26</v>
+      </c>
+      <c r="AB1" t="s">
+        <v>27</v>
+      </c>
+      <c r="AC1" t="s">
+        <v>28</v>
+      </c>
+      <c r="AD1" t="s">
+        <v>29</v>
+      </c>
+      <c r="AE1" t="s">
+        <v>30</v>
+      </c>
+      <c r="AF1" t="s">
+        <v>31</v>
+      </c>
+      <c r="AG1" t="s">
+        <v>32</v>
+      </c>
+      <c r="AH1" t="s">
+        <v>33</v>
+      </c>
+      <c r="AI1" t="s">
+        <v>34</v>
+      </c>
+      <c r="AJ1" t="s">
+        <v>35</v>
+      </c>
+      <c r="AK1" t="s">
+        <v>78</v>
+      </c>
+      <c r="AL1" t="s">
+        <v>79</v>
+      </c>
+      <c r="AM1" t="s">
+        <v>36</v>
+      </c>
+      <c r="AN1" t="s">
+        <v>37</v>
+      </c>
+      <c r="AO1" t="s">
+        <v>38</v>
+      </c>
+      <c r="AP1" t="s">
+        <v>39</v>
+      </c>
+      <c r="AQ1" t="s">
+        <v>40</v>
+      </c>
+      <c r="AR1" t="s">
+        <v>41</v>
+      </c>
+      <c r="AS1" t="s">
+        <v>42</v>
+      </c>
+      <c r="AT1" t="s">
+        <v>43</v>
+      </c>
+      <c r="AU1" t="s">
+        <v>44</v>
+      </c>
+      <c r="AV1" t="s">
+        <v>45</v>
+      </c>
+      <c r="AW1" t="s">
+        <v>46</v>
+      </c>
+      <c r="AX1" t="s">
+        <v>47</v>
+      </c>
+      <c r="AY1" t="s">
+        <v>48</v>
+      </c>
+      <c r="AZ1" t="s">
+        <v>82</v>
+      </c>
+      <c r="BA1" t="s">
+        <v>83</v>
+      </c>
+      <c r="BB1" t="s">
+        <v>84</v>
+      </c>
+      <c r="BC1" t="s">
+        <v>85</v>
+      </c>
+      <c r="BD1" t="s">
+        <v>86</v>
+      </c>
+      <c r="BE1" t="s">
+        <v>87</v>
+      </c>
+      <c r="BF1" t="s">
+        <v>88</v>
+      </c>
+      <c r="BG1" t="s">
+        <v>89</v>
+      </c>
+      <c r="BH1" t="s">
+        <v>90</v>
+      </c>
+      <c r="BI1" t="s">
+        <v>91</v>
+      </c>
+      <c r="BJ1" t="s">
+        <v>92</v>
+      </c>
+      <c r="BK1" t="s">
+        <v>93</v>
+      </c>
+      <c r="BL1" t="s">
+        <v>94</v>
+      </c>
+      <c r="BM1" t="s">
+        <v>95</v>
+      </c>
+      <c r="BN1" t="s">
+        <v>96</v>
+      </c>
+      <c r="BO1" t="s">
+        <v>97</v>
+      </c>
+      <c r="BP1" t="s">
+        <v>98</v>
+      </c>
+      <c r="BQ1" t="s">
+        <v>99</v>
+      </c>
+      <c r="BR1" t="s">
+        <v>100</v>
+      </c>
+      <c r="BS1" t="s">
+        <v>101</v>
+      </c>
+      <c r="BT1" t="s">
+        <v>113</v>
+      </c>
+      <c r="BU1" t="s">
+        <v>114</v>
+      </c>
+      <c r="BV1" t="s">
+        <v>115</v>
+      </c>
+      <c r="BW1" t="s">
+        <v>116</v>
+      </c>
+      <c r="BX1" t="s">
+        <v>117</v>
+      </c>
+      <c r="BY1" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="2" spans="1:77" x14ac:dyDescent="0.2">
+      <c r="A2">
+        <v>11</v>
+      </c>
+      <c r="B2">
+        <v>0</v>
+      </c>
+      <c r="C2">
+        <v>1</v>
+      </c>
+      <c r="D2" t="s">
+        <v>51</v>
+      </c>
+      <c r="E2" t="s">
+        <v>68</v>
+      </c>
+      <c r="F2" t="s">
+        <v>54</v>
+      </c>
+      <c r="G2" t="s">
+        <v>56</v>
+      </c>
+      <c r="H2" t="s">
+        <v>67</v>
+      </c>
+      <c r="I2" t="s">
+        <v>120</v>
+      </c>
+      <c r="J2" t="s">
+        <v>51</v>
+      </c>
+      <c r="K2" t="s">
+        <v>50</v>
+      </c>
+      <c r="M2" t="s">
+        <v>51</v>
+      </c>
+      <c r="N2" t="s">
+        <v>54</v>
+      </c>
+      <c r="O2" t="s">
+        <v>61</v>
+      </c>
+      <c r="P2" t="s">
+        <v>51</v>
+      </c>
+      <c r="Q2" t="s">
+        <v>53</v>
+      </c>
+      <c r="R2" t="s">
+        <v>52</v>
+      </c>
+      <c r="S2" t="s">
+        <v>51</v>
+      </c>
+      <c r="T2" t="s">
+        <v>72</v>
+      </c>
+      <c r="V2" t="s">
+        <v>58</v>
+      </c>
+      <c r="W2" t="s">
+        <v>55</v>
+      </c>
+      <c r="Z2">
+        <v>1</v>
+      </c>
+      <c r="AB2" t="s">
+        <v>67</v>
+      </c>
+      <c r="AC2">
+        <v>1</v>
+      </c>
+      <c r="AD2" t="s">
+        <v>124</v>
+      </c>
+      <c r="AF2" t="s">
+        <v>51</v>
+      </c>
+      <c r="AG2" t="s">
+        <v>58</v>
+      </c>
+      <c r="AH2" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI2" t="s">
+        <v>125</v>
+      </c>
+      <c r="AJ2" t="s">
+        <v>65</v>
+      </c>
+      <c r="AL2" t="s">
+        <v>51</v>
+      </c>
+      <c r="AN2" t="s">
+        <v>51</v>
+      </c>
+      <c r="AO2">
+        <v>1</v>
+      </c>
+      <c r="AP2" t="s">
+        <v>131</v>
+      </c>
+      <c r="AQ2" t="s">
+        <v>51</v>
+      </c>
+      <c r="AR2" t="s">
+        <v>132</v>
+      </c>
+      <c r="AS2">
+        <v>1</v>
+      </c>
+      <c r="AT2">
+        <v>1</v>
+      </c>
+      <c r="AU2" t="s">
+        <v>56</v>
+      </c>
+      <c r="AW2" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="3" spans="1:77" x14ac:dyDescent="0.2">
+      <c r="A3">
+        <v>12</v>
+      </c>
+      <c r="B3">
+        <v>1</v>
+      </c>
+      <c r="C3">
+        <v>1</v>
+      </c>
+      <c r="D3">
+        <v>0</v>
+      </c>
+      <c r="E3" t="s">
+        <v>51</v>
+      </c>
+      <c r="F3" t="s">
+        <v>59</v>
+      </c>
+      <c r="G3">
+        <v>0</v>
+      </c>
+      <c r="H3" t="s">
+        <v>51</v>
+      </c>
+      <c r="I3" t="s">
+        <v>50</v>
+      </c>
+      <c r="J3" t="s">
+        <v>50</v>
+      </c>
+      <c r="K3" t="s">
+        <v>54</v>
+      </c>
+      <c r="L3">
+        <v>1</v>
+      </c>
+      <c r="M3" t="s">
+        <v>49</v>
+      </c>
+      <c r="N3">
+        <v>0</v>
+      </c>
+      <c r="P3" t="s">
+        <v>55</v>
+      </c>
+      <c r="Q3" t="s">
+        <v>68</v>
+      </c>
+      <c r="R3" t="s">
+        <v>51</v>
+      </c>
+      <c r="S3" t="s">
+        <v>54</v>
+      </c>
+      <c r="T3" t="s">
+        <v>51</v>
+      </c>
+      <c r="V3" t="s">
+        <v>51</v>
+      </c>
+      <c r="W3" t="s">
+        <v>58</v>
+      </c>
+      <c r="X3" t="s">
+        <v>50</v>
+      </c>
+      <c r="Y3" t="s">
+        <v>67</v>
+      </c>
+      <c r="Z3" t="s">
+        <v>67</v>
+      </c>
+      <c r="AA3" t="s">
+        <v>72</v>
+      </c>
+      <c r="AB3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AC3" t="s">
+        <v>55</v>
+      </c>
+      <c r="AD3" t="s">
+        <v>126</v>
+      </c>
+      <c r="AE3" t="s">
+        <v>51</v>
+      </c>
+      <c r="AF3" t="s">
+        <v>127</v>
+      </c>
+      <c r="AG3" t="s">
+        <v>49</v>
+      </c>
+      <c r="AH3" t="s">
+        <v>55</v>
+      </c>
+      <c r="AI3" t="s">
+        <v>55</v>
+      </c>
+      <c r="AJ3">
+        <v>1</v>
+      </c>
+      <c r="AL3" t="s">
+        <v>51</v>
+      </c>
+      <c r="AM3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AN3" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="4" spans="1:77" x14ac:dyDescent="0.2">
+      <c r="A4">
+        <v>15</v>
+      </c>
+      <c r="B4">
+        <v>1</v>
+      </c>
+      <c r="C4" t="s">
+        <v>53</v>
+      </c>
+      <c r="D4" t="s">
+        <v>119</v>
+      </c>
+      <c r="E4" t="s">
+        <v>51</v>
+      </c>
+      <c r="F4" t="s">
+        <v>73</v>
+      </c>
+      <c r="G4" t="s">
+        <v>54</v>
+      </c>
+      <c r="H4" t="s">
+        <v>61</v>
+      </c>
+      <c r="I4" t="s">
+        <v>123</v>
+      </c>
+      <c r="L4">
+        <v>0</v>
+      </c>
+      <c r="O4">
+        <v>0</v>
+      </c>
+      <c r="P4">
+        <v>1</v>
+      </c>
+      <c r="R4" t="s">
+        <v>61</v>
+      </c>
+      <c r="S4">
+        <v>1</v>
+      </c>
+      <c r="T4" t="s">
+        <v>60</v>
+      </c>
+      <c r="U4">
+        <v>1</v>
+      </c>
+      <c r="V4" t="s">
+        <v>60</v>
+      </c>
+      <c r="Z4" t="s">
+        <v>60</v>
+      </c>
+      <c r="AB4">
+        <v>0</v>
+      </c>
+      <c r="AC4" t="s">
+        <v>55</v>
+      </c>
+      <c r="AD4">
+        <v>0</v>
+      </c>
+      <c r="AE4" t="s">
+        <v>50</v>
+      </c>
+      <c r="AF4" t="s">
+        <v>55</v>
+      </c>
+      <c r="AG4" t="s">
+        <v>64</v>
+      </c>
+      <c r="AH4" t="s">
+        <v>52</v>
+      </c>
+      <c r="AI4" t="s">
+        <v>59</v>
+      </c>
+      <c r="AJ4" t="s">
+        <v>58</v>
+      </c>
+      <c r="AK4">
+        <v>1</v>
+      </c>
+      <c r="AL4" t="s">
+        <v>49</v>
+      </c>
+      <c r="AM4" t="s">
+        <v>54</v>
+      </c>
+      <c r="AN4" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="5" spans="1:77" x14ac:dyDescent="0.2">
+      <c r="A5">
+        <v>22</v>
+      </c>
+      <c r="B5">
+        <v>0</v>
+      </c>
+      <c r="C5" t="s">
+        <v>50</v>
+      </c>
+      <c r="D5">
+        <v>0</v>
+      </c>
+      <c r="E5" t="s">
+        <v>51</v>
+      </c>
+      <c r="F5" t="s">
+        <v>60</v>
+      </c>
+      <c r="G5" t="s">
+        <v>51</v>
+      </c>
+      <c r="H5">
+        <v>0</v>
+      </c>
+      <c r="I5" t="s">
+        <v>51</v>
+      </c>
+      <c r="J5" t="s">
+        <v>51</v>
+      </c>
+      <c r="K5" t="s">
+        <v>56</v>
+      </c>
+      <c r="L5">
+        <v>1</v>
+      </c>
+      <c r="M5" t="s">
+        <v>60</v>
+      </c>
+      <c r="N5">
+        <v>0</v>
+      </c>
+      <c r="O5">
+        <v>1</v>
+      </c>
+      <c r="P5" t="s">
+        <v>68</v>
+      </c>
+      <c r="Q5" t="s">
+        <v>60</v>
+      </c>
+      <c r="T5">
+        <v>0</v>
+      </c>
+      <c r="Y5">
+        <v>1</v>
+      </c>
+      <c r="AD5">
+        <v>0</v>
+      </c>
+      <c r="AE5">
+        <v>1</v>
+      </c>
+      <c r="AG5">
+        <v>1</v>
+      </c>
+      <c r="AH5" t="s">
+        <v>68</v>
+      </c>
+      <c r="AI5" t="s">
+        <v>51</v>
+      </c>
+      <c r="AJ5">
+        <v>0</v>
+      </c>
+      <c r="AL5">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:77" x14ac:dyDescent="0.2">
+      <c r="A6">
+        <v>31</v>
+      </c>
+      <c r="B6">
+        <v>0</v>
+      </c>
+      <c r="C6" t="s">
+        <v>51</v>
+      </c>
+      <c r="D6" t="s">
+        <v>60</v>
+      </c>
+      <c r="E6" t="s">
+        <v>51</v>
+      </c>
+      <c r="F6" t="s">
+        <v>61</v>
+      </c>
+      <c r="G6" t="s">
+        <v>51</v>
+      </c>
+      <c r="H6">
+        <v>0</v>
+      </c>
+      <c r="I6" t="s">
+        <v>51</v>
+      </c>
+      <c r="J6" t="s">
+        <v>51</v>
+      </c>
+      <c r="K6" t="s">
+        <v>72</v>
+      </c>
+      <c r="L6">
+        <v>1</v>
+      </c>
+      <c r="M6" t="s">
+        <v>49</v>
+      </c>
+      <c r="N6" t="s">
+        <v>60</v>
+      </c>
+      <c r="O6" t="s">
+        <v>51</v>
+      </c>
+      <c r="P6" t="s">
+        <v>68</v>
+      </c>
+      <c r="Q6" t="s">
+        <v>60</v>
+      </c>
+      <c r="V6" t="s">
+        <v>51</v>
+      </c>
+      <c r="W6" t="s">
+        <v>68</v>
+      </c>
+      <c r="X6" t="s">
+        <v>67</v>
+      </c>
+      <c r="Y6" t="s">
+        <v>55</v>
+      </c>
+      <c r="Z6" t="s">
+        <v>55</v>
+      </c>
+      <c r="AA6" t="s">
+        <v>108</v>
+      </c>
+      <c r="AB6" t="s">
+        <v>51</v>
+      </c>
+      <c r="AC6" t="s">
+        <v>51</v>
+      </c>
+      <c r="AD6" t="s">
+        <v>60</v>
+      </c>
+      <c r="AE6">
+        <v>1</v>
+      </c>
+      <c r="AF6" t="s">
+        <v>107</v>
+      </c>
+      <c r="AH6">
+        <v>1</v>
+      </c>
+      <c r="AI6">
+        <v>1</v>
+      </c>
+      <c r="AJ6" t="s">
+        <v>67</v>
+      </c>
+      <c r="AK6" t="s">
+        <v>51</v>
+      </c>
+      <c r="AL6" t="s">
+        <v>77</v>
+      </c>
+      <c r="AN6">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7" spans="1:77" x14ac:dyDescent="0.2">
+      <c r="A7">
+        <v>32</v>
+      </c>
+      <c r="B7" t="s">
+        <v>56</v>
+      </c>
+      <c r="C7" t="s">
+        <v>51</v>
+      </c>
+      <c r="D7">
+        <v>0</v>
+      </c>
+      <c r="F7">
+        <v>0</v>
+      </c>
+      <c r="H7" t="s">
+        <v>62</v>
+      </c>
+      <c r="I7" t="s">
+        <v>53</v>
+      </c>
+      <c r="J7" t="s">
+        <v>53</v>
+      </c>
+      <c r="K7" t="s">
+        <v>77</v>
+      </c>
+      <c r="L7" t="s">
+        <v>49</v>
+      </c>
+      <c r="M7" t="s">
+        <v>110</v>
+      </c>
+      <c r="N7" t="s">
+        <v>80</v>
+      </c>
+      <c r="O7">
+        <v>1</v>
+      </c>
+      <c r="P7" t="s">
+        <v>121</v>
+      </c>
+      <c r="Q7" t="s">
+        <v>122</v>
+      </c>
+      <c r="R7" t="s">
+        <v>53</v>
+      </c>
+      <c r="AB7">
+        <v>1</v>
+      </c>
+      <c r="AC7" t="s">
+        <v>51</v>
+      </c>
+      <c r="AD7" t="s">
+        <v>60</v>
+      </c>
+      <c r="AE7" t="s">
+        <v>53</v>
+      </c>
+      <c r="AF7" t="s">
+        <v>59</v>
+      </c>
+      <c r="AG7" t="s">
+        <v>53</v>
+      </c>
+      <c r="AH7" t="s">
+        <v>121</v>
+      </c>
+      <c r="AI7">
+        <v>1</v>
+      </c>
+      <c r="AJ7" t="s">
+        <v>54</v>
+      </c>
+      <c r="AL7" t="s">
+        <v>50</v>
+      </c>
+      <c r="AM7" t="s">
+        <v>128</v>
+      </c>
+      <c r="AN7" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="8" spans="1:77" x14ac:dyDescent="0.2">
+      <c r="A8">
+        <v>53</v>
+      </c>
+      <c r="B8">
+        <v>0</v>
+      </c>
+      <c r="D8">
+        <v>1</v>
+      </c>
+      <c r="E8" t="s">
+        <v>51</v>
+      </c>
+      <c r="F8" t="s">
+        <v>60</v>
+      </c>
+      <c r="G8">
+        <v>1</v>
+      </c>
+      <c r="H8" t="s">
+        <v>59</v>
+      </c>
+      <c r="I8">
+        <v>1</v>
+      </c>
+      <c r="J8" t="s">
+        <v>51</v>
+      </c>
+      <c r="K8" t="s">
+        <v>68</v>
+      </c>
+      <c r="M8" t="s">
+        <v>60</v>
+      </c>
+      <c r="N8" t="s">
+        <v>55</v>
+      </c>
+      <c r="O8">
+        <v>1</v>
+      </c>
+      <c r="P8" t="s">
+        <v>60</v>
+      </c>
+      <c r="R8" t="s">
+        <v>51</v>
+      </c>
+      <c r="S8" t="s">
+        <v>57</v>
+      </c>
+      <c r="T8" t="s">
+        <v>51</v>
+      </c>
+      <c r="V8" t="s">
+        <v>51</v>
+      </c>
+      <c r="W8" t="s">
+        <v>55</v>
+      </c>
+      <c r="X8" t="s">
+        <v>107</v>
+      </c>
+      <c r="Y8" t="s">
+        <v>54</v>
+      </c>
+      <c r="Z8">
+        <v>1</v>
+      </c>
+      <c r="AA8" t="s">
+        <v>53</v>
+      </c>
+      <c r="AB8" t="s">
+        <v>51</v>
+      </c>
+      <c r="AC8" t="s">
+        <v>51</v>
+      </c>
+      <c r="AD8">
+        <v>1</v>
+      </c>
+      <c r="AE8">
+        <v>1</v>
+      </c>
+      <c r="AF8" t="s">
+        <v>129</v>
+      </c>
+      <c r="AG8" t="s">
+        <v>51</v>
+      </c>
+      <c r="AH8">
+        <v>0</v>
+      </c>
+      <c r="AI8">
+        <v>1</v>
+      </c>
+      <c r="AJ8" t="s">
+        <v>55</v>
+      </c>
+      <c r="AK8" t="s">
+        <v>54</v>
+      </c>
+      <c r="AL8" t="s">
+        <v>72</v>
+      </c>
+      <c r="AM8" t="s">
+        <v>51</v>
+      </c>
+      <c r="AN8" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="9" spans="1:77" x14ac:dyDescent="0.2">
+      <c r="A9">
+        <v>55</v>
+      </c>
+      <c r="B9" t="s">
+        <v>51</v>
+      </c>
+      <c r="C9" t="s">
+        <v>56</v>
+      </c>
+      <c r="E9">
+        <v>0</v>
+      </c>
+      <c r="I9" t="s">
+        <v>68</v>
+      </c>
+      <c r="T9">
+        <v>0</v>
+      </c>
+      <c r="V9" t="s">
+        <v>55</v>
+      </c>
+      <c r="W9" t="s">
+        <v>49</v>
+      </c>
+      <c r="Z9" t="s">
+        <v>51</v>
+      </c>
+      <c r="AC9" t="s">
+        <v>72</v>
+      </c>
+      <c r="AG9" t="s">
+        <v>60</v>
+      </c>
+      <c r="AH9" t="s">
+        <v>130</v>
+      </c>
+      <c r="AI9">
+        <v>1</v>
+      </c>
+      <c r="AJ9" t="s">
+        <v>55</v>
+      </c>
+      <c r="AK9" t="s">
+        <v>55</v>
+      </c>
+      <c r="AM9">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10" spans="1:77" x14ac:dyDescent="0.2">
+      <c r="A10">
+        <v>44</v>
+      </c>
+      <c r="D10">
+        <v>0</v>
+      </c>
+      <c r="E10">
+        <v>0</v>
+      </c>
+      <c r="F10" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="11" spans="1:77" x14ac:dyDescent="0.2">
+      <c r="A11">
+        <v>52</v>
+      </c>
+      <c r="B11">
+        <v>0</v>
+      </c>
+      <c r="C11">
+        <v>1</v>
+      </c>
+      <c r="D11">
+        <v>0</v>
+      </c>
+      <c r="E11">
+        <v>1</v>
+      </c>
+      <c r="F11">
+        <v>0</v>
+      </c>
+      <c r="G11">
+        <v>1</v>
+      </c>
+      <c r="H11" t="s">
+        <v>77</v>
+      </c>
+      <c r="K11" t="s">
+        <v>110</v>
+      </c>
+      <c r="M11" t="s">
+        <v>68</v>
+      </c>
+      <c r="P11" t="s">
+        <v>60</v>
+      </c>
+      <c r="T11" t="s">
+        <v>51</v>
+      </c>
+      <c r="U11" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="12" spans="1:77" x14ac:dyDescent="0.2">
+      <c r="A12">
+        <v>54</v>
+      </c>
+      <c r="C12" t="s">
+        <v>53</v>
+      </c>
+      <c r="D12">
+        <v>0</v>
+      </c>
+      <c r="E12" t="s">
+        <v>51</v>
+      </c>
+      <c r="F12">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{07DD42B4-0D96-BB48-8242-CDEA51D42ED4}">
+  <dimension ref="A1:AL12"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetData>
+    <row r="1" spans="1:38" x14ac:dyDescent="0.2">
+      <c r="A1" t="s">
+        <v>138</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="G1" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="H1" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="I1" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="J1" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="K1" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="L1" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="M1" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="N1" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="O1" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="P1" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="Q1" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="R1" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="S1" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="T1" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="U1" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="V1" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="W1" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="X1" s="2" t="s">
+        <v>82</v>
+      </c>
+      <c r="Y1" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="Z1" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="AA1" s="2" t="s">
+        <v>85</v>
+      </c>
+      <c r="AB1" s="2" t="s">
+        <v>86</v>
+      </c>
+      <c r="AC1" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="AD1" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="AE1" s="2" t="s">
+        <v>89</v>
+      </c>
+      <c r="AF1" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="AG1" s="2" t="s">
+        <v>91</v>
+      </c>
+      <c r="AH1" s="2" t="s">
+        <v>92</v>
+      </c>
+      <c r="AI1" s="2" t="s">
+        <v>93</v>
+      </c>
+      <c r="AJ1" s="2" t="s">
+        <v>94</v>
+      </c>
+      <c r="AK1" s="2" t="s">
+        <v>95</v>
+      </c>
+      <c r="AL1" s="2" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="2" spans="1:38" x14ac:dyDescent="0.2">
+      <c r="A2">
+        <v>11</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>124</v>
+      </c>
+      <c r="C2" s="2"/>
+      <c r="D2" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="F2" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="G2" s="2" t="s">
+        <v>125</v>
+      </c>
+      <c r="H2" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="I2" s="2"/>
+      <c r="J2" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="K2" s="2"/>
+      <c r="L2" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="M2" s="2">
+        <v>1</v>
+      </c>
+      <c r="N2" s="2" t="s">
+        <v>131</v>
+      </c>
+      <c r="O2" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="P2" s="2" t="s">
+        <v>132</v>
+      </c>
+      <c r="Q2" s="2">
+        <v>1</v>
+      </c>
+      <c r="R2" s="2">
+        <v>1</v>
+      </c>
+      <c r="S2" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="T2" s="2"/>
+      <c r="U2" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="V2" s="2"/>
+      <c r="W2" s="2"/>
+      <c r="X2" s="2">
+        <v>1</v>
+      </c>
+      <c r="Y2" s="2">
+        <v>1</v>
+      </c>
+      <c r="Z2" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="AA2" s="2"/>
+      <c r="AB2" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="AC2" s="2"/>
+      <c r="AD2" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="AE2" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="AF2" s="2">
+        <v>1</v>
+      </c>
+      <c r="AG2" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="AH2" s="2"/>
+      <c r="AI2" s="2"/>
+      <c r="AJ2" s="2"/>
+      <c r="AK2" s="2"/>
+      <c r="AL2" s="2"/>
+    </row>
+    <row r="3" spans="1:38" x14ac:dyDescent="0.2">
+      <c r="A3">
+        <v>12</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>126</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>127</v>
+      </c>
+      <c r="E3" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="F3" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="G3" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="H3" s="2">
+        <v>1</v>
+      </c>
+      <c r="I3" s="2"/>
+      <c r="J3" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="K3" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="L3" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="M3" s="2">
+        <v>1</v>
+      </c>
+      <c r="N3" s="2"/>
+      <c r="O3" s="2"/>
+      <c r="P3" s="2"/>
+      <c r="Q3" s="2"/>
+      <c r="R3" s="2"/>
+      <c r="S3" s="2"/>
+      <c r="T3" s="2"/>
+      <c r="U3" s="2"/>
+      <c r="V3" s="2"/>
+      <c r="W3" s="2"/>
+      <c r="X3" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="Y3" s="2">
+        <v>0</v>
+      </c>
+      <c r="Z3" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="AA3" s="2">
+        <v>1</v>
+      </c>
+      <c r="AB3" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="AC3" s="2">
+        <v>0</v>
+      </c>
+      <c r="AD3" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="AE3" s="2" t="s">
+        <v>133</v>
+      </c>
+      <c r="AF3" s="2">
+        <v>1</v>
+      </c>
+      <c r="AG3" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="AH3" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="AI3" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="AJ3" s="2"/>
+      <c r="AK3" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="AL3" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" spans="1:38" x14ac:dyDescent="0.2">
+      <c r="A4">
+        <v>15</v>
+      </c>
+      <c r="B4" s="2">
+        <v>0</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="E4" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="F4" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="G4" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="H4" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="I4" s="2">
+        <v>1</v>
+      </c>
+      <c r="J4" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="K4" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="L4" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="M4" s="2">
+        <v>1</v>
+      </c>
+      <c r="N4" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="O4" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="P4" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="Q4" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="R4" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="S4" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="T4" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="U4" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="V4" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="W4" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="X4" s="2" t="s">
+        <v>134</v>
+      </c>
+      <c r="Y4" s="2">
+        <v>1</v>
+      </c>
+      <c r="Z4" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="AA4" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="AB4" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="AC4" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="AD4" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="AE4" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="AF4" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG4" s="2" t="s">
+        <v>135</v>
+      </c>
+      <c r="AH4" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="AI4" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="AJ4" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="AK4" s="2" t="s">
+        <v>137</v>
+      </c>
+      <c r="AL4" s="2" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="5" spans="1:38" x14ac:dyDescent="0.2">
+      <c r="A5">
+        <v>22</v>
+      </c>
+      <c r="B5" s="2">
+        <v>0</v>
+      </c>
+      <c r="C5" s="2">
+        <v>1</v>
+      </c>
+      <c r="D5" s="2"/>
+      <c r="E5" s="2">
+        <v>1</v>
+      </c>
+      <c r="F5" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="G5" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="H5" s="2">
+        <v>0</v>
+      </c>
+      <c r="I5" s="2"/>
+      <c r="J5" s="2">
+        <v>0</v>
+      </c>
+      <c r="K5" s="2"/>
+      <c r="L5" s="2"/>
+      <c r="M5" s="2"/>
+      <c r="N5" s="2"/>
+      <c r="O5" s="2">
+        <v>0</v>
+      </c>
+      <c r="P5" s="2"/>
+      <c r="Q5" s="2"/>
+      <c r="R5" s="2">
+        <v>1</v>
+      </c>
+      <c r="S5" s="2">
+        <v>1</v>
+      </c>
+      <c r="T5" s="2">
+        <v>0</v>
+      </c>
+      <c r="U5" s="2">
+        <v>0</v>
+      </c>
+      <c r="V5" s="2"/>
+      <c r="W5" s="2">
+        <v>0</v>
+      </c>
+      <c r="X5" s="2">
+        <v>0</v>
+      </c>
+      <c r="Y5" s="2">
+        <v>1</v>
+      </c>
+      <c r="Z5" s="2"/>
+      <c r="AA5" s="2"/>
+      <c r="AB5" s="2">
+        <v>0</v>
+      </c>
+      <c r="AC5" s="2">
+        <v>1</v>
+      </c>
+      <c r="AD5" s="2">
+        <v>0</v>
+      </c>
+      <c r="AE5" s="2"/>
+      <c r="AF5" s="2">
+        <v>0</v>
+      </c>
+      <c r="AG5" s="2">
+        <v>1</v>
+      </c>
+      <c r="AH5" s="2">
+        <v>0</v>
+      </c>
+      <c r="AI5" s="2">
+        <v>1</v>
+      </c>
+      <c r="AJ5" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="AK5" s="2"/>
+      <c r="AL5" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:38" x14ac:dyDescent="0.2">
+      <c r="A6">
+        <v>31</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="C6" s="2">
+        <v>1</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="E6" s="2"/>
+      <c r="F6" s="2">
+        <v>1</v>
+      </c>
+      <c r="G6" s="2">
+        <v>1</v>
+      </c>
+      <c r="H6" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="I6" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="J6" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="K6" s="2"/>
+      <c r="L6" s="2">
+        <v>1</v>
+      </c>
+      <c r="M6" s="2">
+        <v>0</v>
+      </c>
+      <c r="N6" s="2"/>
+      <c r="O6" s="2"/>
+      <c r="P6" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="Q6" s="2">
+        <v>0</v>
+      </c>
+      <c r="R6" s="2">
+        <v>0</v>
+      </c>
+      <c r="S6" s="2">
+        <v>1</v>
+      </c>
+      <c r="T6" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="U6" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="V6" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="W6" s="2" t="s">
+        <v>133</v>
+      </c>
+      <c r="X6" s="2" t="s">
+        <v>126</v>
+      </c>
+      <c r="Y6" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="Z6" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="AA6" s="2"/>
+      <c r="AB6" s="2"/>
+      <c r="AC6" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="AD6" s="2" t="s">
+        <v>110</v>
+      </c>
+      <c r="AE6" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="AF6" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="AG6" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="AH6" s="2"/>
+      <c r="AI6" s="2"/>
+      <c r="AJ6" s="2"/>
+      <c r="AK6" s="2"/>
+      <c r="AL6" s="2"/>
+    </row>
+    <row r="7" spans="1:38" x14ac:dyDescent="0.2">
+      <c r="A7">
+        <v>32</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="D7" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="E7" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="F7" s="2" t="s">
+        <v>121</v>
+      </c>
+      <c r="G7" s="2">
+        <v>1</v>
+      </c>
+      <c r="H7" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="I7" s="2"/>
+      <c r="J7" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="K7" s="2" t="s">
+        <v>128</v>
+      </c>
+      <c r="L7" s="2" t="s">
+        <v>102</v>
+      </c>
+      <c r="M7" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="N7" s="2"/>
+      <c r="O7" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="P7" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="Q7" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="R7" s="2">
+        <v>1</v>
+      </c>
+      <c r="S7" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="T7" s="2" t="s">
+        <v>134</v>
+      </c>
+      <c r="U7" s="2">
+        <v>0</v>
+      </c>
+      <c r="V7" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="W7" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="X7" s="2"/>
+      <c r="Y7" s="2"/>
+      <c r="Z7" s="2"/>
+      <c r="AA7" s="2"/>
+      <c r="AB7" s="2"/>
+      <c r="AC7" s="2"/>
+      <c r="AD7" s="2"/>
+      <c r="AE7" s="2"/>
+      <c r="AF7" s="2"/>
+      <c r="AG7" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="AH7" s="2"/>
+      <c r="AI7" s="2">
+        <v>1</v>
+      </c>
+      <c r="AJ7" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="AK7" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="AL7" s="2" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="8" spans="1:38" x14ac:dyDescent="0.2">
+      <c r="A8">
+        <v>53</v>
+      </c>
+      <c r="B8" s="2">
+        <v>1</v>
+      </c>
+      <c r="C8" s="2">
+        <v>1</v>
+      </c>
+      <c r="D8" s="2" t="s">
+        <v>129</v>
+      </c>
+      <c r="E8" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="F8" s="2">
+        <v>0</v>
+      </c>
+      <c r="G8" s="2">
+        <v>1</v>
+      </c>
+      <c r="H8" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="I8" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="J8" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="K8" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="L8" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="M8" s="2"/>
+      <c r="N8" s="2"/>
+      <c r="O8" s="2"/>
+      <c r="P8" s="2"/>
+      <c r="Q8" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="R8" s="2"/>
+      <c r="S8" s="2"/>
+      <c r="T8" s="2"/>
+      <c r="U8" s="2"/>
+      <c r="V8" s="2"/>
+      <c r="W8" s="2"/>
+      <c r="X8" s="2"/>
+      <c r="Y8" s="2"/>
+      <c r="Z8" s="2"/>
+      <c r="AA8" s="2"/>
+      <c r="AB8" s="2"/>
+      <c r="AC8" s="2">
+        <v>1</v>
+      </c>
+      <c r="AD8" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="AE8" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="AF8" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="AG8" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="AH8" s="2"/>
+      <c r="AI8" s="2">
+        <v>1</v>
+      </c>
+      <c r="AJ8" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="AK8" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="AL8" s="2" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="9" spans="1:38" x14ac:dyDescent="0.2">
+      <c r="A9">
+        <v>55</v>
+      </c>
+      <c r="B9" s="2"/>
+      <c r="C9" s="2"/>
+      <c r="D9" s="2"/>
+      <c r="E9" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="F9" s="2" t="s">
+        <v>130</v>
+      </c>
+      <c r="G9" s="2">
+        <v>1</v>
+      </c>
+      <c r="H9" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="I9" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="J9" s="2"/>
+      <c r="K9" s="2">
+        <v>1</v>
+      </c>
+      <c r="L9" s="2"/>
+      <c r="M9" s="2">
+        <v>1</v>
+      </c>
+      <c r="N9" s="2"/>
+      <c r="O9" s="2"/>
+      <c r="P9" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="Q9" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="R9" s="2">
+        <v>0</v>
+      </c>
+      <c r="S9" s="2">
+        <v>0</v>
+      </c>
+      <c r="T9" s="2"/>
+      <c r="U9" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="V9" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="W9" s="2"/>
+      <c r="X9" s="2">
+        <v>1</v>
+      </c>
+      <c r="Y9" s="2">
+        <v>0</v>
+      </c>
+      <c r="Z9" s="2"/>
+      <c r="AA9" s="2">
+        <v>1</v>
+      </c>
+      <c r="AB9" s="2"/>
+      <c r="AC9" s="2">
+        <v>0</v>
+      </c>
+      <c r="AD9" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="AE9" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="AF9" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="AG9" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="AH9" s="2">
+        <v>1</v>
+      </c>
+      <c r="AI9" s="2">
+        <v>0</v>
+      </c>
+      <c r="AJ9" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="AK9" s="2"/>
+      <c r="AL9" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10" spans="1:38" x14ac:dyDescent="0.2">
+      <c r="A10">
+        <v>44</v>
+      </c>
+      <c r="B10" s="2"/>
+      <c r="C10" s="2"/>
+      <c r="D10" s="2"/>
+      <c r="E10" s="2"/>
+      <c r="F10" s="2"/>
+      <c r="G10" s="2"/>
+      <c r="H10" s="2"/>
+      <c r="I10" s="2"/>
+      <c r="J10" s="2"/>
+      <c r="K10" s="2"/>
+      <c r="L10" s="2"/>
+      <c r="M10" s="2"/>
+      <c r="N10" s="2"/>
+      <c r="O10" s="2"/>
+      <c r="P10" s="2"/>
+      <c r="Q10" s="2"/>
+      <c r="R10" s="2"/>
+      <c r="S10" s="2"/>
+      <c r="T10" s="2"/>
+      <c r="U10" s="2"/>
+      <c r="V10" s="2"/>
+      <c r="W10" s="2"/>
+      <c r="X10" s="2"/>
+      <c r="Y10" s="2"/>
+      <c r="Z10" s="2"/>
+      <c r="AA10" s="2"/>
+      <c r="AB10" s="2"/>
+      <c r="AC10" s="2"/>
+      <c r="AD10" s="2"/>
+      <c r="AE10" s="2"/>
+      <c r="AF10" s="2"/>
+      <c r="AG10" s="2"/>
+      <c r="AH10" s="2"/>
+      <c r="AI10" s="2"/>
+      <c r="AJ10" s="2"/>
+      <c r="AK10" s="2"/>
+      <c r="AL10" s="2"/>
+    </row>
+    <row r="11" spans="1:38" x14ac:dyDescent="0.2">
+      <c r="A11">
+        <v>52</v>
+      </c>
+      <c r="B11" s="2"/>
+      <c r="C11" s="2"/>
+      <c r="D11" s="2"/>
+      <c r="E11" s="2"/>
+      <c r="F11" s="2"/>
+      <c r="G11" s="2"/>
+      <c r="H11" s="2"/>
+      <c r="I11" s="2"/>
+      <c r="J11" s="2"/>
+      <c r="K11" s="2"/>
+      <c r="L11" s="2"/>
+      <c r="M11" s="2"/>
+      <c r="N11" s="2"/>
+      <c r="O11" s="2"/>
+      <c r="P11" s="2"/>
+      <c r="Q11" s="2"/>
+      <c r="R11" s="2"/>
+      <c r="S11" s="2"/>
+      <c r="T11" s="2"/>
+      <c r="U11" s="2"/>
+      <c r="V11" s="2"/>
+      <c r="W11" s="2"/>
+      <c r="X11" s="2"/>
+      <c r="Y11" s="2"/>
+      <c r="Z11" s="2"/>
+      <c r="AA11" s="2"/>
+      <c r="AB11" s="2"/>
+      <c r="AC11" s="2"/>
+      <c r="AD11" s="2"/>
+      <c r="AE11" s="2"/>
+      <c r="AF11" s="2"/>
+      <c r="AG11" s="2"/>
+      <c r="AH11" s="2"/>
+      <c r="AI11" s="2"/>
+      <c r="AJ11" s="2"/>
+      <c r="AK11" s="2"/>
+      <c r="AL11" s="2"/>
+    </row>
+    <row r="12" spans="1:38" x14ac:dyDescent="0.2">
+      <c r="A12">
+        <v>54</v>
+      </c>
+      <c r="B12" s="2"/>
+      <c r="C12" s="2"/>
+      <c r="D12" s="2"/>
+      <c r="E12" s="2"/>
+      <c r="F12" s="2"/>
+      <c r="G12" s="2"/>
+      <c r="H12" s="2"/>
+      <c r="I12" s="2"/>
+      <c r="J12" s="2"/>
+      <c r="K12" s="2"/>
+      <c r="L12" s="2"/>
+      <c r="M12" s="2"/>
+      <c r="N12" s="2"/>
+      <c r="O12" s="2"/>
+      <c r="P12" s="2"/>
+      <c r="Q12" s="2"/>
+      <c r="R12" s="2"/>
+      <c r="S12" s="2"/>
+      <c r="T12" s="2"/>
+      <c r="U12" s="2"/>
+      <c r="V12" s="2"/>
+      <c r="W12" s="2"/>
+      <c r="X12" s="2"/>
+      <c r="Y12" s="2"/>
+      <c r="Z12" s="2"/>
+      <c r="AA12" s="2"/>
+      <c r="AB12" s="2"/>
+      <c r="AC12" s="2"/>
+      <c r="AD12" s="2"/>
+      <c r="AE12" s="2"/>
+      <c r="AF12" s="2"/>
+      <c r="AG12" s="2"/>
+      <c r="AH12" s="2"/>
+      <c r="AI12" s="2"/>
+      <c r="AJ12" s="2"/>
+      <c r="AK12" s="2"/>
+      <c r="AL12" s="2"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FA71E746-83F5-D346-A573-89DD5E2F0800}">
+  <dimension ref="A1:L12"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetData>
+    <row r="1" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>98</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>99</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>100</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>101</v>
+      </c>
+      <c r="G1" s="2" t="s">
+        <v>113</v>
+      </c>
+      <c r="H1" s="2" t="s">
+        <v>114</v>
+      </c>
+      <c r="I1" s="2" t="s">
+        <v>115</v>
+      </c>
+      <c r="J1" s="2" t="s">
+        <v>116</v>
+      </c>
+      <c r="K1" s="2" t="s">
+        <v>117</v>
+      </c>
+      <c r="L1" s="2" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="2" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A2">
+        <v>11</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="C2" s="2">
+        <v>1</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>136</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="F2" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="G2" s="2">
+        <v>0</v>
+      </c>
+      <c r="H2" s="2" t="s">
+        <v>106</v>
+      </c>
+      <c r="I2" s="2"/>
+      <c r="J2" s="2"/>
+      <c r="K2" s="2"/>
+      <c r="L2" s="2"/>
+    </row>
+    <row r="3" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A3">
+        <v>12</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="C3" s="2">
+        <v>1</v>
+      </c>
+      <c r="D3" s="2"/>
+      <c r="E3" s="2">
+        <v>1</v>
+      </c>
+      <c r="F3" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="G3" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="H3" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="I3" s="2"/>
+      <c r="J3" s="2"/>
+      <c r="K3" s="2"/>
+      <c r="L3" s="2"/>
+    </row>
+    <row r="4" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A4">
+        <v>15</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="C4" s="2"/>
+      <c r="D4" s="2"/>
+      <c r="E4" s="2">
+        <v>1</v>
+      </c>
+      <c r="F4" s="2">
+        <v>1</v>
+      </c>
+      <c r="G4" s="2">
+        <v>1</v>
+      </c>
+      <c r="H4" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="I4" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="J4" s="2">
+        <v>1</v>
+      </c>
+      <c r="K4" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="L4" s="2" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="5" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A5">
+        <v>22</v>
+      </c>
+      <c r="B5" s="2"/>
+      <c r="C5" s="2"/>
+      <c r="D5" s="2"/>
+      <c r="E5" s="2">
+        <v>0</v>
+      </c>
+      <c r="F5" s="2"/>
+      <c r="G5" s="2">
+        <v>0</v>
+      </c>
+      <c r="H5" s="2">
+        <v>1</v>
+      </c>
+      <c r="I5" s="2">
+        <v>0</v>
+      </c>
+      <c r="J5" s="2"/>
+      <c r="K5" s="2"/>
+      <c r="L5" s="2"/>
+    </row>
+    <row r="6" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A6">
+        <v>31</v>
+      </c>
+      <c r="B6" s="2"/>
+      <c r="C6" s="2"/>
+      <c r="D6" s="2"/>
+      <c r="E6" s="2">
+        <v>0</v>
+      </c>
+      <c r="F6" s="2"/>
+      <c r="G6" s="2">
+        <v>1</v>
+      </c>
+      <c r="H6" s="2"/>
+      <c r="I6" s="2"/>
+      <c r="J6" s="2"/>
+      <c r="K6" s="2"/>
+      <c r="L6" s="2"/>
+    </row>
+    <row r="7" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A7">
+        <v>32</v>
+      </c>
+      <c r="B7" s="2"/>
+      <c r="C7" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="D7" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="E7" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="F7" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="G7" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="H7" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="I7" s="2">
+        <v>0</v>
+      </c>
+      <c r="J7" s="2">
+        <v>1</v>
+      </c>
+      <c r="K7" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="L7" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A8">
+        <v>53</v>
+      </c>
+      <c r="B8" s="2"/>
+      <c r="C8" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="D8" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="E8" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="F8" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="G8" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="H8" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="I8" s="2">
+        <v>1</v>
+      </c>
+      <c r="J8" s="2"/>
+      <c r="K8" s="2"/>
+      <c r="L8" s="2"/>
+    </row>
+    <row r="9" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A9">
+        <v>55</v>
+      </c>
+      <c r="B9" s="2"/>
+      <c r="C9" s="2"/>
+      <c r="D9" s="2">
+        <v>0</v>
+      </c>
+      <c r="E9" s="2"/>
+      <c r="F9" s="2">
+        <v>0</v>
+      </c>
+      <c r="G9" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="H9" s="2">
+        <v>0</v>
+      </c>
+      <c r="I9" s="2">
+        <v>1</v>
+      </c>
+      <c r="J9" s="2"/>
+      <c r="K9" s="2"/>
+      <c r="L9" s="2"/>
+    </row>
+    <row r="10" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A10">
+        <v>44</v>
+      </c>
+      <c r="B10" s="2"/>
+      <c r="C10" s="2"/>
+      <c r="D10" s="2"/>
+      <c r="E10" s="2"/>
+      <c r="F10" s="2"/>
+      <c r="G10" s="2"/>
+      <c r="H10" s="2"/>
+      <c r="I10" s="2"/>
+      <c r="J10" s="2"/>
+      <c r="K10" s="2"/>
+      <c r="L10" s="2"/>
+    </row>
+    <row r="11" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A11">
+        <v>52</v>
+      </c>
+      <c r="B11" s="2"/>
+      <c r="C11" s="2"/>
+      <c r="D11" s="2"/>
+      <c r="E11" s="2"/>
+      <c r="F11" s="2"/>
+      <c r="G11" s="2"/>
+      <c r="H11" s="2"/>
+      <c r="I11" s="2"/>
+      <c r="J11" s="2"/>
+      <c r="K11" s="2"/>
+      <c r="L11" s="2"/>
+    </row>
+    <row r="12" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A12">
+        <v>54</v>
+      </c>
+      <c r="B12" s="2"/>
+      <c r="C12" s="2"/>
+      <c r="D12" s="2"/>
+      <c r="E12" s="2"/>
+      <c r="F12" s="2"/>
+      <c r="G12" s="2"/>
+      <c r="H12" s="2"/>
+      <c r="I12" s="2"/>
+      <c r="J12" s="2"/>
+      <c r="K12" s="2"/>
+      <c r="L12" s="2"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Before Claude session - safety snapshot
</commit_message>
<xml_diff>
--- a/data/raw/2025/data_summer_2025.xlsx
+++ b/data/raw/2025/data_summer_2025.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10720"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10727"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://lunduniversityo365-my.sharepoint.com/personal/an4718sc_lu_se/Documents/PhD/projects/dorsal_snapshot_discrimination_project/analysis/data/raw/2025/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="563" documentId="8_{BAD0E982-56D3-0E41-B109-60B516BAC403}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5F871857-CC79-8647-A291-636AC4A09480}"/>
+  <xr:revisionPtr revIDLastSave="1522" documentId="8_{BAD0E982-56D3-0E41-B109-60B516BAC403}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8B2B3E15-3DF4-A54F-9439-0CDF1B31792B}"/>
   <bookViews>
-    <workbookView xWindow="4240" yWindow="2020" windowWidth="28040" windowHeight="17440" activeTab="2" xr2:uid="{0F60F085-ABCE-EA48-9AAF-DAFB43BA76C4}"/>
+    <workbookView xWindow="4240" yWindow="2020" windowWidth="28040" windowHeight="17440" activeTab="9" xr2:uid="{0F60F085-ABCE-EA48-9AAF-DAFB43BA76C4}"/>
   </bookViews>
   <sheets>
     <sheet name="170725" sheetId="1" r:id="rId1"/>
@@ -19,6 +19,10 @@
     <sheet name="300725_natcan" sheetId="4" r:id="rId4"/>
     <sheet name="310725natcan" sheetId="5" r:id="rId5"/>
     <sheet name="010825natcan" sheetId="6" r:id="rId6"/>
+    <sheet name="080825_natcan_3D" sheetId="7" r:id="rId7"/>
+    <sheet name="090825_natcan_3D" sheetId="8" r:id="rId8"/>
+    <sheet name="090825_natcan_3D_ctrl" sheetId="9" r:id="rId9"/>
+    <sheet name="250725_brightness_diff" sheetId="10" r:id="rId10"/>
   </sheets>
   <calcPr calcId="181029"/>
   <extLst>
@@ -41,7 +45,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="904" uniqueCount="139">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1562" uniqueCount="224">
   <si>
     <t>individual</t>
   </si>
@@ -457,7 +461,262 @@
     <t>0,1,0,0,0,0,1</t>
   </si>
   <si>
-    <t xml:space="preserve">  </t>
+    <t>6L</t>
+  </si>
+  <si>
+    <t>7R</t>
+  </si>
+  <si>
+    <t>9L</t>
+  </si>
+  <si>
+    <t>11L</t>
+  </si>
+  <si>
+    <t>10R</t>
+  </si>
+  <si>
+    <t>13R</t>
+  </si>
+  <si>
+    <t>14L</t>
+  </si>
+  <si>
+    <t>16R</t>
+  </si>
+  <si>
+    <t>17L</t>
+  </si>
+  <si>
+    <t>20R</t>
+  </si>
+  <si>
+    <t>21L</t>
+  </si>
+  <si>
+    <t>23R</t>
+  </si>
+  <si>
+    <t>24L</t>
+  </si>
+  <si>
+    <t>26R</t>
+  </si>
+  <si>
+    <t>28L</t>
+  </si>
+  <si>
+    <t>29R</t>
+  </si>
+  <si>
+    <t>30L</t>
+  </si>
+  <si>
+    <t>31R</t>
+  </si>
+  <si>
+    <t>32L</t>
+  </si>
+  <si>
+    <t>33R</t>
+  </si>
+  <si>
+    <t>34L</t>
+  </si>
+  <si>
+    <t>35R</t>
+  </si>
+  <si>
+    <t>36L</t>
+  </si>
+  <si>
+    <t>37R</t>
+  </si>
+  <si>
+    <t>38L</t>
+  </si>
+  <si>
+    <t>40R</t>
+  </si>
+  <si>
+    <t>41L</t>
+  </si>
+  <si>
+    <t>42R</t>
+  </si>
+  <si>
+    <t>43L</t>
+  </si>
+  <si>
+    <t>44R</t>
+  </si>
+  <si>
+    <t>46L</t>
+  </si>
+  <si>
+    <t>48R</t>
+  </si>
+  <si>
+    <t>49L</t>
+  </si>
+  <si>
+    <t>51R</t>
+  </si>
+  <si>
+    <t>53L</t>
+  </si>
+  <si>
+    <t>55R</t>
+  </si>
+  <si>
+    <t>56L</t>
+  </si>
+  <si>
+    <t>57R</t>
+  </si>
+  <si>
+    <t>58L</t>
+  </si>
+  <si>
+    <t>59R</t>
+  </si>
+  <si>
+    <t>60L</t>
+  </si>
+  <si>
+    <t>61R</t>
+  </si>
+  <si>
+    <t>62L</t>
+  </si>
+  <si>
+    <t>63R</t>
+  </si>
+  <si>
+    <t>64L</t>
+  </si>
+  <si>
+    <t>65R</t>
+  </si>
+  <si>
+    <t>66L</t>
+  </si>
+  <si>
+    <t>67R</t>
+  </si>
+  <si>
+    <t>68L</t>
+  </si>
+  <si>
+    <t>69R</t>
+  </si>
+  <si>
+    <t>70L</t>
+  </si>
+  <si>
+    <t>71R</t>
+  </si>
+  <si>
+    <t>72L</t>
+  </si>
+  <si>
+    <t>73R</t>
+  </si>
+  <si>
+    <t>74L</t>
+  </si>
+  <si>
+    <t>77L</t>
+  </si>
+  <si>
+    <t>78R</t>
+  </si>
+  <si>
+    <t>79L</t>
+  </si>
+  <si>
+    <t>80L</t>
+  </si>
+  <si>
+    <t>81R</t>
+  </si>
+  <si>
+    <t>82R</t>
+  </si>
+  <si>
+    <t>83L</t>
+  </si>
+  <si>
+    <t>84R</t>
+  </si>
+  <si>
+    <t>85L</t>
+  </si>
+  <si>
+    <t>86L</t>
+  </si>
+  <si>
+    <t>87R</t>
+  </si>
+  <si>
+    <t>88L</t>
+  </si>
+  <si>
+    <t>89R</t>
+  </si>
+  <si>
+    <t>90R</t>
+  </si>
+  <si>
+    <t>91L</t>
+  </si>
+  <si>
+    <t>92R</t>
+  </si>
+  <si>
+    <t>93L</t>
+  </si>
+  <si>
+    <t>94R</t>
+  </si>
+  <si>
+    <t>0,0,0,1,1,0</t>
+  </si>
+  <si>
+    <t>0,0,0,1,0</t>
+  </si>
+  <si>
+    <t>0,0,1,0,0</t>
+  </si>
+  <si>
+    <t>0,0,0,0,0,0,0,0,1</t>
+  </si>
+  <si>
+    <t>0,0,1,1,1</t>
+  </si>
+  <si>
+    <t>0,0,0,0,1,0,0</t>
+  </si>
+  <si>
+    <t>0,0,0,0,1,0,0,0</t>
+  </si>
+  <si>
+    <t>1,0,0,0,0</t>
+  </si>
+  <si>
+    <t>0,0,0,0,0,0,0,0,0,0,0,0</t>
+  </si>
+  <si>
+    <t>1,0,0,0,0,1</t>
+  </si>
+  <si>
+    <t>0,0,0,1,1</t>
+  </si>
+  <si>
+    <t>0,0,0,0,0,0,0,0,0,0,0,0,0</t>
+  </si>
+  <si>
+    <t>,0,1</t>
   </si>
 </sst>
 </file>
@@ -1318,6 +1577,455 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F0DE98AA-E79C-7142-8A2A-44E60000BF87}">
+  <dimension ref="A1:AC8"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetData>
+    <row r="1" spans="1:29" x14ac:dyDescent="0.2">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" t="s">
+        <v>9</v>
+      </c>
+      <c r="K1" t="s">
+        <v>10</v>
+      </c>
+      <c r="L1" t="s">
+        <v>11</v>
+      </c>
+      <c r="M1" t="s">
+        <v>12</v>
+      </c>
+      <c r="N1" t="s">
+        <v>143</v>
+      </c>
+      <c r="O1" t="s">
+        <v>14</v>
+      </c>
+      <c r="P1" t="s">
+        <v>15</v>
+      </c>
+      <c r="Q1" t="s">
+        <v>145</v>
+      </c>
+      <c r="R1" t="s">
+        <v>17</v>
+      </c>
+      <c r="S1" t="s">
+        <v>111</v>
+      </c>
+      <c r="T1" t="s">
+        <v>112</v>
+      </c>
+      <c r="U1" t="s">
+        <v>20</v>
+      </c>
+      <c r="V1" t="s">
+        <v>21</v>
+      </c>
+      <c r="W1" t="s">
+        <v>22</v>
+      </c>
+      <c r="X1" t="s">
+        <v>23</v>
+      </c>
+      <c r="Y1" t="s">
+        <v>24</v>
+      </c>
+      <c r="Z1" t="s">
+        <v>25</v>
+      </c>
+      <c r="AA1" t="s">
+        <v>26</v>
+      </c>
+      <c r="AB1" t="s">
+        <v>27</v>
+      </c>
+      <c r="AC1" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="2" spans="1:29" x14ac:dyDescent="0.2">
+      <c r="A2">
+        <v>12</v>
+      </c>
+      <c r="B2" t="s">
+        <v>51</v>
+      </c>
+      <c r="C2">
+        <v>0</v>
+      </c>
+      <c r="D2" t="s">
+        <v>54</v>
+      </c>
+      <c r="E2" t="s">
+        <v>50</v>
+      </c>
+      <c r="F2" t="s">
+        <v>54</v>
+      </c>
+      <c r="G2" t="s">
+        <v>72</v>
+      </c>
+      <c r="I2" t="s">
+        <v>51</v>
+      </c>
+      <c r="J2" t="s">
+        <v>51</v>
+      </c>
+      <c r="K2" t="s">
+        <v>51</v>
+      </c>
+      <c r="L2" t="s">
+        <v>53</v>
+      </c>
+      <c r="M2" t="s">
+        <v>51</v>
+      </c>
+      <c r="N2" t="s">
+        <v>51</v>
+      </c>
+      <c r="O2" t="s">
+        <v>50</v>
+      </c>
+      <c r="P2" t="s">
+        <v>51</v>
+      </c>
+      <c r="Q2" t="s">
+        <v>51</v>
+      </c>
+      <c r="R2" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="3" spans="1:29" x14ac:dyDescent="0.2">
+      <c r="A3">
+        <v>13</v>
+      </c>
+      <c r="B3">
+        <v>0</v>
+      </c>
+      <c r="C3">
+        <v>1</v>
+      </c>
+      <c r="D3" t="s">
+        <v>68</v>
+      </c>
+      <c r="E3" t="s">
+        <v>51</v>
+      </c>
+      <c r="F3" t="s">
+        <v>77</v>
+      </c>
+      <c r="G3">
+        <v>1</v>
+      </c>
+      <c r="I3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" spans="1:29" x14ac:dyDescent="0.2">
+      <c r="A4">
+        <v>22</v>
+      </c>
+      <c r="B4" t="s">
+        <v>55</v>
+      </c>
+      <c r="D4" t="s">
+        <v>60</v>
+      </c>
+      <c r="E4" t="s">
+        <v>55</v>
+      </c>
+      <c r="F4" t="s">
+        <v>59</v>
+      </c>
+      <c r="G4">
+        <v>1</v>
+      </c>
+      <c r="I4">
+        <v>1</v>
+      </c>
+      <c r="J4" t="s">
+        <v>51</v>
+      </c>
+      <c r="K4">
+        <v>1</v>
+      </c>
+      <c r="L4" t="s">
+        <v>51</v>
+      </c>
+      <c r="M4">
+        <v>1</v>
+      </c>
+      <c r="N4" t="s">
+        <v>51</v>
+      </c>
+      <c r="O4" t="s">
+        <v>51</v>
+      </c>
+      <c r="P4" t="s">
+        <v>51</v>
+      </c>
+      <c r="Q4" t="s">
+        <v>51</v>
+      </c>
+      <c r="R4">
+        <v>1</v>
+      </c>
+      <c r="S4">
+        <v>0</v>
+      </c>
+      <c r="T4" t="s">
+        <v>51</v>
+      </c>
+      <c r="U4" t="s">
+        <v>49</v>
+      </c>
+      <c r="V4" t="s">
+        <v>51</v>
+      </c>
+      <c r="W4" t="s">
+        <v>61</v>
+      </c>
+      <c r="X4" t="s">
+        <v>58</v>
+      </c>
+      <c r="Y4" t="s">
+        <v>51</v>
+      </c>
+      <c r="Z4" t="s">
+        <v>53</v>
+      </c>
+      <c r="AA4" t="s">
+        <v>51</v>
+      </c>
+      <c r="AB4" t="s">
+        <v>68</v>
+      </c>
+      <c r="AC4" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="5" spans="1:29" x14ac:dyDescent="0.2">
+      <c r="A5">
+        <v>23</v>
+      </c>
+      <c r="B5">
+        <v>1</v>
+      </c>
+      <c r="C5" t="s">
+        <v>49</v>
+      </c>
+      <c r="D5">
+        <v>1</v>
+      </c>
+      <c r="F5" t="s">
+        <v>60</v>
+      </c>
+      <c r="G5">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6" spans="1:29" x14ac:dyDescent="0.2">
+      <c r="A6">
+        <v>33</v>
+      </c>
+      <c r="B6" t="s">
+        <v>51</v>
+      </c>
+      <c r="C6" t="s">
+        <v>68</v>
+      </c>
+      <c r="D6" t="s">
+        <v>51</v>
+      </c>
+      <c r="E6" t="s">
+        <v>77</v>
+      </c>
+      <c r="F6">
+        <v>1</v>
+      </c>
+      <c r="G6">
+        <v>0</v>
+      </c>
+      <c r="K6" t="s">
+        <v>51</v>
+      </c>
+      <c r="L6" t="s">
+        <v>68</v>
+      </c>
+      <c r="O6">
+        <v>0</v>
+      </c>
+      <c r="P6" t="s">
+        <v>49</v>
+      </c>
+      <c r="Q6" t="s">
+        <v>58</v>
+      </c>
+      <c r="R6" t="s">
+        <v>53</v>
+      </c>
+      <c r="S6">
+        <v>1</v>
+      </c>
+      <c r="T6" t="s">
+        <v>56</v>
+      </c>
+      <c r="U6" t="s">
+        <v>51</v>
+      </c>
+      <c r="V6" t="s">
+        <v>54</v>
+      </c>
+      <c r="W6">
+        <v>1</v>
+      </c>
+      <c r="X6" t="s">
+        <v>51</v>
+      </c>
+      <c r="Y6" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="7" spans="1:29" x14ac:dyDescent="0.2">
+      <c r="A7">
+        <v>44</v>
+      </c>
+      <c r="B7" t="s">
+        <v>51</v>
+      </c>
+      <c r="C7" t="s">
+        <v>49</v>
+      </c>
+      <c r="D7" t="s">
+        <v>54</v>
+      </c>
+      <c r="E7" t="s">
+        <v>81</v>
+      </c>
+      <c r="F7">
+        <v>1</v>
+      </c>
+      <c r="G7" t="s">
+        <v>68</v>
+      </c>
+      <c r="H7">
+        <v>1</v>
+      </c>
+      <c r="I7" t="s">
+        <v>68</v>
+      </c>
+      <c r="J7" t="s">
+        <v>77</v>
+      </c>
+      <c r="K7" t="s">
+        <v>51</v>
+      </c>
+      <c r="L7" t="s">
+        <v>68</v>
+      </c>
+      <c r="M7" t="s">
+        <v>51</v>
+      </c>
+      <c r="N7" t="s">
+        <v>68</v>
+      </c>
+      <c r="O7" t="s">
+        <v>68</v>
+      </c>
+      <c r="P7" t="s">
+        <v>51</v>
+      </c>
+      <c r="Q7" t="s">
+        <v>68</v>
+      </c>
+      <c r="R7" t="s">
+        <v>218</v>
+      </c>
+    </row>
+    <row r="8" spans="1:29" x14ac:dyDescent="0.2">
+      <c r="A8">
+        <v>53</v>
+      </c>
+      <c r="B8">
+        <v>1</v>
+      </c>
+      <c r="C8" t="s">
+        <v>60</v>
+      </c>
+      <c r="D8" t="s">
+        <v>51</v>
+      </c>
+      <c r="E8" t="s">
+        <v>54</v>
+      </c>
+      <c r="F8" t="s">
+        <v>54</v>
+      </c>
+      <c r="I8">
+        <v>1</v>
+      </c>
+      <c r="J8">
+        <v>1</v>
+      </c>
+      <c r="K8">
+        <v>0</v>
+      </c>
+      <c r="L8" t="s">
+        <v>51</v>
+      </c>
+      <c r="M8" t="s">
+        <v>56</v>
+      </c>
+      <c r="N8" t="s">
+        <v>55</v>
+      </c>
+      <c r="O8" t="s">
+        <v>51</v>
+      </c>
+      <c r="P8" t="s">
+        <v>51</v>
+      </c>
+      <c r="Q8" t="s">
+        <v>51</v>
+      </c>
+      <c r="R8" t="s">
+        <v>51</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{73A9D138-CAA1-8846-8EBE-E8765EC1A531}">
   <dimension ref="A1:AJ10"/>
@@ -3516,7 +4224,7 @@
   <sheetData>
     <row r="1" spans="1:38" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
-        <v>138</v>
+        <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
         <v>29</v>
@@ -4833,4 +5541,2320 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{277EABA8-1B46-8B42-A3A6-CBC36CD222A6}">
+  <dimension ref="A1:AS11"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetData>
+    <row r="1" spans="1:45" x14ac:dyDescent="0.2">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" t="s">
+        <v>138</v>
+      </c>
+      <c r="H1" t="s">
+        <v>139</v>
+      </c>
+      <c r="I1" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" t="s">
+        <v>140</v>
+      </c>
+      <c r="K1" t="s">
+        <v>142</v>
+      </c>
+      <c r="L1" t="s">
+        <v>141</v>
+      </c>
+      <c r="M1" t="s">
+        <v>12</v>
+      </c>
+      <c r="N1" t="s">
+        <v>143</v>
+      </c>
+      <c r="O1" t="s">
+        <v>144</v>
+      </c>
+      <c r="P1" t="s">
+        <v>15</v>
+      </c>
+      <c r="Q1" t="s">
+        <v>145</v>
+      </c>
+      <c r="R1" t="s">
+        <v>146</v>
+      </c>
+      <c r="S1" t="s">
+        <v>18</v>
+      </c>
+      <c r="T1" t="s">
+        <v>19</v>
+      </c>
+      <c r="U1" t="s">
+        <v>147</v>
+      </c>
+      <c r="V1" t="s">
+        <v>148</v>
+      </c>
+      <c r="W1" t="s">
+        <v>22</v>
+      </c>
+      <c r="X1" t="s">
+        <v>149</v>
+      </c>
+      <c r="Y1" t="s">
+        <v>150</v>
+      </c>
+      <c r="Z1" t="s">
+        <v>25</v>
+      </c>
+      <c r="AA1" t="s">
+        <v>151</v>
+      </c>
+      <c r="AB1" t="s">
+        <v>27</v>
+      </c>
+      <c r="AC1" t="s">
+        <v>152</v>
+      </c>
+      <c r="AD1" t="s">
+        <v>153</v>
+      </c>
+      <c r="AE1" t="s">
+        <v>154</v>
+      </c>
+      <c r="AF1" t="s">
+        <v>155</v>
+      </c>
+      <c r="AG1" t="s">
+        <v>156</v>
+      </c>
+      <c r="AH1" t="s">
+        <v>157</v>
+      </c>
+      <c r="AI1" t="s">
+        <v>158</v>
+      </c>
+      <c r="AJ1" t="s">
+        <v>159</v>
+      </c>
+      <c r="AK1" t="s">
+        <v>160</v>
+      </c>
+      <c r="AL1" t="s">
+        <v>161</v>
+      </c>
+      <c r="AM1" t="s">
+        <v>162</v>
+      </c>
+      <c r="AN1" t="s">
+        <v>37</v>
+      </c>
+      <c r="AO1" t="s">
+        <v>163</v>
+      </c>
+      <c r="AP1" t="s">
+        <v>164</v>
+      </c>
+      <c r="AQ1" t="s">
+        <v>165</v>
+      </c>
+      <c r="AR1" t="s">
+        <v>166</v>
+      </c>
+      <c r="AS1" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="2" spans="1:45" x14ac:dyDescent="0.2">
+      <c r="A2">
+        <v>11</v>
+      </c>
+      <c r="B2">
+        <v>1</v>
+      </c>
+      <c r="C2" t="s">
+        <v>49</v>
+      </c>
+      <c r="D2" t="s">
+        <v>52</v>
+      </c>
+      <c r="E2">
+        <v>1</v>
+      </c>
+      <c r="F2" t="s">
+        <v>51</v>
+      </c>
+      <c r="G2" t="s">
+        <v>60</v>
+      </c>
+      <c r="H2" t="s">
+        <v>51</v>
+      </c>
+      <c r="I2" t="s">
+        <v>51</v>
+      </c>
+      <c r="J2" t="s">
+        <v>56</v>
+      </c>
+      <c r="K2" t="s">
+        <v>51</v>
+      </c>
+      <c r="L2" t="s">
+        <v>81</v>
+      </c>
+      <c r="M2" t="s">
+        <v>129</v>
+      </c>
+      <c r="N2" t="s">
+        <v>51</v>
+      </c>
+      <c r="O2" t="s">
+        <v>77</v>
+      </c>
+      <c r="P2" t="s">
+        <v>81</v>
+      </c>
+      <c r="Q2">
+        <v>1</v>
+      </c>
+      <c r="R2" t="s">
+        <v>57</v>
+      </c>
+      <c r="S2" t="s">
+        <v>51</v>
+      </c>
+      <c r="T2" t="s">
+        <v>56</v>
+      </c>
+      <c r="W2" t="s">
+        <v>58</v>
+      </c>
+      <c r="X2" t="s">
+        <v>51</v>
+      </c>
+      <c r="Y2" t="s">
+        <v>106</v>
+      </c>
+      <c r="Z2" t="s">
+        <v>58</v>
+      </c>
+      <c r="AA2" t="s">
+        <v>51</v>
+      </c>
+      <c r="AB2">
+        <v>1</v>
+      </c>
+      <c r="AE2" t="s">
+        <v>55</v>
+      </c>
+      <c r="AF2" t="s">
+        <v>51</v>
+      </c>
+      <c r="AG2" t="s">
+        <v>58</v>
+      </c>
+      <c r="AH2" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI2" t="s">
+        <v>51</v>
+      </c>
+      <c r="AJ2" t="s">
+        <v>53</v>
+      </c>
+      <c r="AL2">
+        <v>1</v>
+      </c>
+      <c r="AM2">
+        <v>1</v>
+      </c>
+      <c r="AN2" t="s">
+        <v>51</v>
+      </c>
+      <c r="AO2" t="s">
+        <v>55</v>
+      </c>
+      <c r="AQ2">
+        <v>1</v>
+      </c>
+      <c r="AR2" t="s">
+        <v>60</v>
+      </c>
+      <c r="AS2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:45" x14ac:dyDescent="0.2">
+      <c r="A3">
+        <v>12</v>
+      </c>
+      <c r="B3" t="s">
+        <v>60</v>
+      </c>
+      <c r="C3">
+        <v>1</v>
+      </c>
+      <c r="D3" t="s">
+        <v>60</v>
+      </c>
+      <c r="E3">
+        <v>1</v>
+      </c>
+      <c r="F3" t="s">
+        <v>49</v>
+      </c>
+      <c r="G3">
+        <v>0</v>
+      </c>
+      <c r="H3" t="s">
+        <v>60</v>
+      </c>
+      <c r="I3" t="s">
+        <v>49</v>
+      </c>
+      <c r="J3" t="s">
+        <v>51</v>
+      </c>
+      <c r="L3">
+        <v>1</v>
+      </c>
+      <c r="M3" t="s">
+        <v>51</v>
+      </c>
+      <c r="N3" t="s">
+        <v>211</v>
+      </c>
+      <c r="O3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P3" t="s">
+        <v>51</v>
+      </c>
+      <c r="Q3" t="s">
+        <v>60</v>
+      </c>
+      <c r="R3" t="s">
+        <v>51</v>
+      </c>
+      <c r="S3" t="s">
+        <v>58</v>
+      </c>
+      <c r="U3">
+        <v>0</v>
+      </c>
+      <c r="X3">
+        <v>0</v>
+      </c>
+      <c r="Y3">
+        <v>1</v>
+      </c>
+      <c r="AA3" t="s">
+        <v>60</v>
+      </c>
+      <c r="AH3">
+        <v>0</v>
+      </c>
+      <c r="AR3">
+        <v>1</v>
+      </c>
+      <c r="AS3" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="4" spans="1:45" x14ac:dyDescent="0.2">
+      <c r="A4">
+        <v>13</v>
+      </c>
+      <c r="B4" t="s">
+        <v>49</v>
+      </c>
+      <c r="C4" t="s">
+        <v>72</v>
+      </c>
+      <c r="D4" t="s">
+        <v>51</v>
+      </c>
+      <c r="E4" t="s">
+        <v>54</v>
+      </c>
+      <c r="F4" t="s">
+        <v>58</v>
+      </c>
+      <c r="G4" t="s">
+        <v>54</v>
+      </c>
+      <c r="H4" t="s">
+        <v>53</v>
+      </c>
+      <c r="I4" t="s">
+        <v>63</v>
+      </c>
+      <c r="J4" t="s">
+        <v>127</v>
+      </c>
+      <c r="K4" t="s">
+        <v>60</v>
+      </c>
+      <c r="L4" t="s">
+        <v>51</v>
+      </c>
+      <c r="M4" t="s">
+        <v>127</v>
+      </c>
+      <c r="N4">
+        <v>1</v>
+      </c>
+      <c r="O4" t="s">
+        <v>58</v>
+      </c>
+      <c r="P4" t="s">
+        <v>50</v>
+      </c>
+      <c r="Q4" t="s">
+        <v>56</v>
+      </c>
+      <c r="R4" t="s">
+        <v>51</v>
+      </c>
+      <c r="S4" t="s">
+        <v>72</v>
+      </c>
+      <c r="T4">
+        <v>1</v>
+      </c>
+      <c r="U4" t="s">
+        <v>61</v>
+      </c>
+      <c r="V4" t="s">
+        <v>49</v>
+      </c>
+      <c r="W4" t="s">
+        <v>49</v>
+      </c>
+      <c r="X4" t="s">
+        <v>49</v>
+      </c>
+      <c r="Y4" t="s">
+        <v>51</v>
+      </c>
+      <c r="Z4" t="s">
+        <v>54</v>
+      </c>
+      <c r="AA4" t="s">
+        <v>62</v>
+      </c>
+      <c r="AB4" t="s">
+        <v>67</v>
+      </c>
+      <c r="AC4" t="s">
+        <v>67</v>
+      </c>
+      <c r="AD4" t="s">
+        <v>55</v>
+      </c>
+      <c r="AE4" t="s">
+        <v>110</v>
+      </c>
+      <c r="AK4">
+        <v>1</v>
+      </c>
+      <c r="AN4">
+        <v>1</v>
+      </c>
+      <c r="AS4">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" spans="1:45" x14ac:dyDescent="0.2">
+      <c r="A5">
+        <v>15</v>
+      </c>
+      <c r="C5" t="s">
+        <v>60</v>
+      </c>
+      <c r="D5">
+        <v>0</v>
+      </c>
+      <c r="G5" t="s">
+        <v>60</v>
+      </c>
+      <c r="M5">
+        <v>1</v>
+      </c>
+      <c r="O5">
+        <v>0</v>
+      </c>
+      <c r="Q5">
+        <v>1</v>
+      </c>
+      <c r="R5">
+        <v>1</v>
+      </c>
+      <c r="V5">
+        <v>0</v>
+      </c>
+      <c r="W5" t="s">
+        <v>55</v>
+      </c>
+      <c r="AH5">
+        <v>0</v>
+      </c>
+      <c r="AI5" t="s">
+        <v>60</v>
+      </c>
+      <c r="AK5">
+        <v>0</v>
+      </c>
+      <c r="AL5" t="s">
+        <v>68</v>
+      </c>
+      <c r="AM5">
+        <v>1</v>
+      </c>
+      <c r="AN5" t="s">
+        <v>55</v>
+      </c>
+      <c r="AO5" t="s">
+        <v>60</v>
+      </c>
+      <c r="AP5">
+        <v>1</v>
+      </c>
+      <c r="AQ5" t="s">
+        <v>60</v>
+      </c>
+      <c r="AR5">
+        <v>1</v>
+      </c>
+      <c r="AS5" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="6" spans="1:45" x14ac:dyDescent="0.2">
+      <c r="A6">
+        <v>22</v>
+      </c>
+      <c r="B6" t="s">
+        <v>55</v>
+      </c>
+      <c r="C6" t="s">
+        <v>68</v>
+      </c>
+      <c r="D6" t="s">
+        <v>51</v>
+      </c>
+      <c r="E6" t="s">
+        <v>132</v>
+      </c>
+      <c r="F6" t="s">
+        <v>69</v>
+      </c>
+      <c r="G6" t="s">
+        <v>53</v>
+      </c>
+      <c r="H6" t="s">
+        <v>57</v>
+      </c>
+      <c r="I6" t="s">
+        <v>77</v>
+      </c>
+      <c r="J6" t="s">
+        <v>51</v>
+      </c>
+      <c r="K6" t="s">
+        <v>68</v>
+      </c>
+      <c r="L6" t="s">
+        <v>53</v>
+      </c>
+      <c r="M6" t="s">
+        <v>51</v>
+      </c>
+      <c r="N6" t="s">
+        <v>121</v>
+      </c>
+      <c r="O6" t="s">
+        <v>51</v>
+      </c>
+      <c r="P6" t="s">
+        <v>71</v>
+      </c>
+      <c r="Q6" t="s">
+        <v>68</v>
+      </c>
+      <c r="S6" t="s">
+        <v>80</v>
+      </c>
+      <c r="T6" t="s">
+        <v>51</v>
+      </c>
+      <c r="U6" t="s">
+        <v>212</v>
+      </c>
+      <c r="V6">
+        <v>1</v>
+      </c>
+      <c r="W6">
+        <v>1</v>
+      </c>
+      <c r="X6" t="s">
+        <v>212</v>
+      </c>
+      <c r="Y6" t="s">
+        <v>53</v>
+      </c>
+      <c r="Z6">
+        <v>1</v>
+      </c>
+      <c r="AA6" t="s">
+        <v>213</v>
+      </c>
+      <c r="AB6" t="s">
+        <v>56</v>
+      </c>
+      <c r="AC6" t="s">
+        <v>51</v>
+      </c>
+      <c r="AD6" t="s">
+        <v>72</v>
+      </c>
+      <c r="AE6" t="s">
+        <v>51</v>
+      </c>
+      <c r="AF6" t="s">
+        <v>106</v>
+      </c>
+      <c r="AG6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AH6" t="s">
+        <v>215</v>
+      </c>
+      <c r="AI6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AJ6" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="7" spans="1:45" x14ac:dyDescent="0.2">
+      <c r="A7">
+        <v>23</v>
+      </c>
+      <c r="B7">
+        <v>1</v>
+      </c>
+      <c r="C7" t="s">
+        <v>68</v>
+      </c>
+      <c r="D7">
+        <v>1</v>
+      </c>
+      <c r="E7" t="s">
+        <v>55</v>
+      </c>
+      <c r="F7">
+        <v>1</v>
+      </c>
+      <c r="G7">
+        <v>1</v>
+      </c>
+      <c r="H7" t="s">
+        <v>60</v>
+      </c>
+      <c r="K7" t="s">
+        <v>56</v>
+      </c>
+      <c r="L7">
+        <v>1</v>
+      </c>
+      <c r="M7" t="s">
+        <v>51</v>
+      </c>
+      <c r="N7" t="s">
+        <v>68</v>
+      </c>
+      <c r="O7">
+        <v>1</v>
+      </c>
+      <c r="P7" t="s">
+        <v>51</v>
+      </c>
+      <c r="Q7" t="s">
+        <v>58</v>
+      </c>
+      <c r="R7" t="s">
+        <v>51</v>
+      </c>
+      <c r="S7" t="s">
+        <v>81</v>
+      </c>
+      <c r="T7">
+        <v>0</v>
+      </c>
+      <c r="W7">
+        <v>1</v>
+      </c>
+      <c r="X7" t="s">
+        <v>60</v>
+      </c>
+      <c r="Y7">
+        <v>1</v>
+      </c>
+      <c r="Z7" t="s">
+        <v>51</v>
+      </c>
+      <c r="AA7" t="s">
+        <v>129</v>
+      </c>
+      <c r="AB7" t="s">
+        <v>77</v>
+      </c>
+      <c r="AC7">
+        <v>1</v>
+      </c>
+      <c r="AD7" t="s">
+        <v>72</v>
+      </c>
+      <c r="AE7">
+        <v>1</v>
+      </c>
+      <c r="AF7" t="s">
+        <v>59</v>
+      </c>
+      <c r="AG7" t="s">
+        <v>53</v>
+      </c>
+      <c r="AH7" t="s">
+        <v>121</v>
+      </c>
+      <c r="AI7">
+        <v>1</v>
+      </c>
+      <c r="AJ7" t="s">
+        <v>56</v>
+      </c>
+      <c r="AK7">
+        <v>1</v>
+      </c>
+      <c r="AL7" t="s">
+        <v>72</v>
+      </c>
+      <c r="AM7">
+        <v>1</v>
+      </c>
+      <c r="AN7" t="s">
+        <v>51</v>
+      </c>
+      <c r="AP7">
+        <v>1</v>
+      </c>
+      <c r="AQ7" t="s">
+        <v>81</v>
+      </c>
+      <c r="AR7" t="s">
+        <v>51</v>
+      </c>
+      <c r="AS7" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="8" spans="1:45" x14ac:dyDescent="0.2">
+      <c r="A8">
+        <v>25</v>
+      </c>
+      <c r="B8" t="s">
+        <v>51</v>
+      </c>
+      <c r="C8" t="s">
+        <v>59</v>
+      </c>
+      <c r="D8" t="s">
+        <v>53</v>
+      </c>
+      <c r="E8" t="s">
+        <v>52</v>
+      </c>
+      <c r="F8" t="s">
+        <v>63</v>
+      </c>
+      <c r="G8" t="s">
+        <v>67</v>
+      </c>
+      <c r="H8" t="s">
+        <v>59</v>
+      </c>
+      <c r="I8" t="s">
+        <v>60</v>
+      </c>
+      <c r="J8">
+        <v>1</v>
+      </c>
+      <c r="K8" t="s">
+        <v>58</v>
+      </c>
+      <c r="L8" t="s">
+        <v>51</v>
+      </c>
+      <c r="M8" t="s">
+        <v>51</v>
+      </c>
+      <c r="N8" t="s">
+        <v>75</v>
+      </c>
+      <c r="O8" t="s">
+        <v>66</v>
+      </c>
+      <c r="P8" t="s">
+        <v>50</v>
+      </c>
+      <c r="Q8" t="s">
+        <v>54</v>
+      </c>
+      <c r="R8" t="s">
+        <v>51</v>
+      </c>
+      <c r="S8" t="s">
+        <v>51</v>
+      </c>
+      <c r="U8">
+        <v>1</v>
+      </c>
+      <c r="V8">
+        <v>1</v>
+      </c>
+      <c r="W8" t="s">
+        <v>55</v>
+      </c>
+      <c r="X8" t="s">
+        <v>56</v>
+      </c>
+      <c r="Y8" t="s">
+        <v>51</v>
+      </c>
+      <c r="Z8" t="s">
+        <v>51</v>
+      </c>
+      <c r="AA8" t="s">
+        <v>129</v>
+      </c>
+      <c r="AB8" t="s">
+        <v>51</v>
+      </c>
+      <c r="AJ8" t="s">
+        <v>60</v>
+      </c>
+      <c r="AK8" t="s">
+        <v>51</v>
+      </c>
+      <c r="AL8" t="s">
+        <v>216</v>
+      </c>
+      <c r="AN8" t="s">
+        <v>51</v>
+      </c>
+      <c r="AO8" t="s">
+        <v>50</v>
+      </c>
+      <c r="AQ8" t="s">
+        <v>58</v>
+      </c>
+      <c r="AR8" t="s">
+        <v>51</v>
+      </c>
+      <c r="AS8" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="9" spans="1:45" x14ac:dyDescent="0.2">
+      <c r="A9">
+        <v>33</v>
+      </c>
+      <c r="C9">
+        <v>0</v>
+      </c>
+      <c r="E9">
+        <v>1</v>
+      </c>
+      <c r="H9">
+        <v>1</v>
+      </c>
+      <c r="J9">
+        <v>1</v>
+      </c>
+      <c r="K9">
+        <v>0</v>
+      </c>
+      <c r="M9">
+        <v>1</v>
+      </c>
+      <c r="N9" t="s">
+        <v>51</v>
+      </c>
+      <c r="O9" t="s">
+        <v>50</v>
+      </c>
+      <c r="P9" t="s">
+        <v>54</v>
+      </c>
+      <c r="Q9" t="s">
+        <v>52</v>
+      </c>
+      <c r="R9" t="s">
+        <v>102</v>
+      </c>
+      <c r="T9">
+        <v>1</v>
+      </c>
+      <c r="U9" t="s">
+        <v>59</v>
+      </c>
+      <c r="V9" t="s">
+        <v>51</v>
+      </c>
+      <c r="W9" t="s">
+        <v>51</v>
+      </c>
+      <c r="X9" t="s">
+        <v>58</v>
+      </c>
+      <c r="Y9" t="s">
+        <v>53</v>
+      </c>
+      <c r="Z9">
+        <v>1</v>
+      </c>
+      <c r="AA9" t="s">
+        <v>51</v>
+      </c>
+      <c r="AB9" t="s">
+        <v>69</v>
+      </c>
+      <c r="AC9">
+        <v>1</v>
+      </c>
+      <c r="AD9" t="s">
+        <v>68</v>
+      </c>
+      <c r="AE9">
+        <v>1</v>
+      </c>
+      <c r="AF9" t="s">
+        <v>50</v>
+      </c>
+      <c r="AG9" t="s">
+        <v>51</v>
+      </c>
+      <c r="AH9" t="s">
+        <v>58</v>
+      </c>
+      <c r="AI9" t="s">
+        <v>51</v>
+      </c>
+      <c r="AJ9" t="s">
+        <v>51</v>
+      </c>
+      <c r="AM9" t="s">
+        <v>51</v>
+      </c>
+      <c r="AN9" t="s">
+        <v>51</v>
+      </c>
+      <c r="AO9" t="s">
+        <v>77</v>
+      </c>
+      <c r="AP9" t="s">
+        <v>51</v>
+      </c>
+      <c r="AQ9" t="s">
+        <v>129</v>
+      </c>
+      <c r="AS9" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="10" spans="1:45" x14ac:dyDescent="0.2">
+      <c r="A10">
+        <v>35</v>
+      </c>
+      <c r="B10">
+        <v>0</v>
+      </c>
+      <c r="C10">
+        <v>1</v>
+      </c>
+      <c r="D10" t="s">
+        <v>55</v>
+      </c>
+      <c r="E10" t="s">
+        <v>51</v>
+      </c>
+      <c r="F10" t="s">
+        <v>55</v>
+      </c>
+      <c r="G10" t="s">
+        <v>133</v>
+      </c>
+      <c r="H10" t="s">
+        <v>49</v>
+      </c>
+      <c r="I10" t="s">
+        <v>51</v>
+      </c>
+      <c r="J10" t="s">
+        <v>68</v>
+      </c>
+      <c r="K10">
+        <v>1</v>
+      </c>
+      <c r="L10" t="s">
+        <v>68</v>
+      </c>
+      <c r="M10" t="s">
+        <v>129</v>
+      </c>
+      <c r="N10">
+        <v>1</v>
+      </c>
+      <c r="O10" t="s">
+        <v>67</v>
+      </c>
+      <c r="P10">
+        <v>1</v>
+      </c>
+      <c r="Q10">
+        <v>0</v>
+      </c>
+      <c r="R10">
+        <v>0</v>
+      </c>
+      <c r="S10">
+        <v>1</v>
+      </c>
+      <c r="U10">
+        <v>1</v>
+      </c>
+      <c r="V10" t="s">
+        <v>60</v>
+      </c>
+      <c r="X10">
+        <v>1</v>
+      </c>
+      <c r="Y10" t="s">
+        <v>214</v>
+      </c>
+      <c r="Z10" t="s">
+        <v>106</v>
+      </c>
+      <c r="AA10">
+        <v>1</v>
+      </c>
+      <c r="AB10" t="s">
+        <v>51</v>
+      </c>
+      <c r="AD10">
+        <v>1</v>
+      </c>
+      <c r="AF10" t="s">
+        <v>51</v>
+      </c>
+      <c r="AG10" t="s">
+        <v>57</v>
+      </c>
+      <c r="AH10">
+        <v>1</v>
+      </c>
+      <c r="AI10" t="s">
+        <v>129</v>
+      </c>
+      <c r="AK10" t="s">
+        <v>60</v>
+      </c>
+      <c r="AN10">
+        <v>1</v>
+      </c>
+      <c r="AO10" t="s">
+        <v>51</v>
+      </c>
+      <c r="AR10" t="s">
+        <v>49</v>
+      </c>
+      <c r="AS10" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="11" spans="1:45" x14ac:dyDescent="0.2">
+      <c r="A11">
+        <v>55</v>
+      </c>
+      <c r="B11" t="s">
+        <v>55</v>
+      </c>
+      <c r="C11" t="s">
+        <v>50</v>
+      </c>
+      <c r="D11" t="s">
+        <v>64</v>
+      </c>
+      <c r="E11" t="s">
+        <v>50</v>
+      </c>
+      <c r="F11" t="s">
+        <v>50</v>
+      </c>
+      <c r="G11" t="s">
+        <v>51</v>
+      </c>
+      <c r="H11" t="s">
+        <v>107</v>
+      </c>
+      <c r="I11" t="s">
+        <v>54</v>
+      </c>
+      <c r="J11" t="s">
+        <v>51</v>
+      </c>
+      <c r="K11" t="s">
+        <v>55</v>
+      </c>
+      <c r="L11">
+        <v>1</v>
+      </c>
+      <c r="R11" t="s">
+        <v>51</v>
+      </c>
+      <c r="S11">
+        <v>1</v>
+      </c>
+      <c r="V11">
+        <v>1</v>
+      </c>
+      <c r="Y11">
+        <v>1</v>
+      </c>
+      <c r="AC11">
+        <v>1</v>
+      </c>
+      <c r="AN11">
+        <v>1</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A954BAC6-D2D8-6C4A-9998-D0739D57CB2D}">
+  <dimension ref="A1:AE11"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetData>
+    <row r="1" spans="1:31" x14ac:dyDescent="0.2">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>43</v>
+      </c>
+      <c r="C1" t="s">
+        <v>168</v>
+      </c>
+      <c r="D1" t="s">
+        <v>45</v>
+      </c>
+      <c r="E1" t="s">
+        <v>169</v>
+      </c>
+      <c r="F1" t="s">
+        <v>170</v>
+      </c>
+      <c r="G1" t="s">
+        <v>48</v>
+      </c>
+      <c r="H1" t="s">
+        <v>171</v>
+      </c>
+      <c r="I1" t="s">
+        <v>83</v>
+      </c>
+      <c r="J1" t="s">
+        <v>172</v>
+      </c>
+      <c r="K1" t="s">
+        <v>85</v>
+      </c>
+      <c r="L1" t="s">
+        <v>173</v>
+      </c>
+      <c r="M1" t="s">
+        <v>174</v>
+      </c>
+      <c r="N1" t="s">
+        <v>175</v>
+      </c>
+      <c r="O1" t="s">
+        <v>176</v>
+      </c>
+      <c r="P1" t="s">
+        <v>177</v>
+      </c>
+      <c r="Q1" t="s">
+        <v>178</v>
+      </c>
+      <c r="R1" t="s">
+        <v>179</v>
+      </c>
+      <c r="S1" t="s">
+        <v>180</v>
+      </c>
+      <c r="T1" t="s">
+        <v>181</v>
+      </c>
+      <c r="U1" t="s">
+        <v>182</v>
+      </c>
+      <c r="V1" t="s">
+        <v>183</v>
+      </c>
+      <c r="W1" t="s">
+        <v>184</v>
+      </c>
+      <c r="X1" t="s">
+        <v>185</v>
+      </c>
+      <c r="Y1" t="s">
+        <v>186</v>
+      </c>
+      <c r="Z1" t="s">
+        <v>187</v>
+      </c>
+      <c r="AA1" t="s">
+        <v>188</v>
+      </c>
+      <c r="AB1" t="s">
+        <v>189</v>
+      </c>
+      <c r="AC1" t="s">
+        <v>190</v>
+      </c>
+      <c r="AD1" t="s">
+        <v>191</v>
+      </c>
+      <c r="AE1" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="2" spans="1:31" x14ac:dyDescent="0.2">
+      <c r="A2">
+        <v>11</v>
+      </c>
+      <c r="F2" t="s">
+        <v>56</v>
+      </c>
+      <c r="G2">
+        <v>0</v>
+      </c>
+      <c r="H2" t="s">
+        <v>51</v>
+      </c>
+      <c r="I2">
+        <v>1</v>
+      </c>
+      <c r="J2" t="s">
+        <v>56</v>
+      </c>
+      <c r="K2" t="s">
+        <v>58</v>
+      </c>
+      <c r="L2" t="s">
+        <v>53</v>
+      </c>
+      <c r="M2" t="s">
+        <v>57</v>
+      </c>
+      <c r="N2" t="s">
+        <v>51</v>
+      </c>
+      <c r="O2">
+        <v>1</v>
+      </c>
+      <c r="P2" t="s">
+        <v>51</v>
+      </c>
+      <c r="Q2" t="s">
+        <v>57</v>
+      </c>
+      <c r="R2" t="s">
+        <v>51</v>
+      </c>
+      <c r="S2" t="s">
+        <v>60</v>
+      </c>
+      <c r="U2" t="s">
+        <v>68</v>
+      </c>
+      <c r="V2">
+        <v>1</v>
+      </c>
+      <c r="W2">
+        <v>1</v>
+      </c>
+      <c r="X2" t="s">
+        <v>51</v>
+      </c>
+      <c r="Y2" t="s">
+        <v>61</v>
+      </c>
+      <c r="Z2" t="s">
+        <v>51</v>
+      </c>
+      <c r="AA2" t="s">
+        <v>106</v>
+      </c>
+      <c r="AB2">
+        <v>1</v>
+      </c>
+      <c r="AC2" t="s">
+        <v>67</v>
+      </c>
+      <c r="AD2" t="s">
+        <v>53</v>
+      </c>
+      <c r="AE2" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="3" spans="1:31" x14ac:dyDescent="0.2">
+      <c r="A3">
+        <v>12</v>
+      </c>
+      <c r="B3" t="s">
+        <v>77</v>
+      </c>
+      <c r="C3" t="s">
+        <v>51</v>
+      </c>
+      <c r="D3" t="s">
+        <v>54</v>
+      </c>
+      <c r="E3" t="s">
+        <v>68</v>
+      </c>
+      <c r="F3">
+        <v>1</v>
+      </c>
+      <c r="G3" t="s">
+        <v>51</v>
+      </c>
+      <c r="H3" t="s">
+        <v>55</v>
+      </c>
+      <c r="I3" t="s">
+        <v>67</v>
+      </c>
+      <c r="J3" t="s">
+        <v>50</v>
+      </c>
+      <c r="K3" t="s">
+        <v>51</v>
+      </c>
+      <c r="L3" t="s">
+        <v>68</v>
+      </c>
+      <c r="N3">
+        <v>0</v>
+      </c>
+      <c r="R3">
+        <v>0</v>
+      </c>
+      <c r="T3" t="s">
+        <v>60</v>
+      </c>
+      <c r="U3">
+        <v>1</v>
+      </c>
+      <c r="V3" t="s">
+        <v>81</v>
+      </c>
+      <c r="W3" t="s">
+        <v>49</v>
+      </c>
+      <c r="X3" t="s">
+        <v>60</v>
+      </c>
+      <c r="Y3" t="s">
+        <v>55</v>
+      </c>
+      <c r="Z3">
+        <v>0</v>
+      </c>
+      <c r="AB3" t="s">
+        <v>68</v>
+      </c>
+      <c r="AD3" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="4" spans="1:31" x14ac:dyDescent="0.2">
+      <c r="A4">
+        <v>13</v>
+      </c>
+      <c r="M4">
+        <v>0</v>
+      </c>
+      <c r="N4">
+        <v>1</v>
+      </c>
+      <c r="O4" t="s">
+        <v>133</v>
+      </c>
+      <c r="P4">
+        <v>1</v>
+      </c>
+      <c r="V4" t="s">
+        <v>60</v>
+      </c>
+      <c r="W4">
+        <v>1</v>
+      </c>
+      <c r="X4">
+        <v>1</v>
+      </c>
+      <c r="Z4" t="s">
+        <v>55</v>
+      </c>
+      <c r="AA4" t="s">
+        <v>67</v>
+      </c>
+      <c r="AB4" t="s">
+        <v>51</v>
+      </c>
+      <c r="AC4" t="s">
+        <v>51</v>
+      </c>
+      <c r="AD4" t="s">
+        <v>67</v>
+      </c>
+      <c r="AE4" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="5" spans="1:31" x14ac:dyDescent="0.2">
+      <c r="A5">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="6" spans="1:31" x14ac:dyDescent="0.2">
+      <c r="A6">
+        <v>22</v>
+      </c>
+      <c r="B6">
+        <v>1</v>
+      </c>
+      <c r="C6" t="s">
+        <v>51</v>
+      </c>
+      <c r="D6" t="s">
+        <v>53</v>
+      </c>
+      <c r="E6" t="s">
+        <v>62</v>
+      </c>
+      <c r="F6">
+        <v>1</v>
+      </c>
+      <c r="G6" t="s">
+        <v>51</v>
+      </c>
+      <c r="H6" t="s">
+        <v>50</v>
+      </c>
+      <c r="I6" t="s">
+        <v>58</v>
+      </c>
+      <c r="J6" t="s">
+        <v>51</v>
+      </c>
+      <c r="K6" t="s">
+        <v>53</v>
+      </c>
+      <c r="L6" t="s">
+        <v>128</v>
+      </c>
+      <c r="M6" t="s">
+        <v>71</v>
+      </c>
+      <c r="N6" t="s">
+        <v>51</v>
+      </c>
+      <c r="O6" t="s">
+        <v>53</v>
+      </c>
+      <c r="P6" t="s">
+        <v>69</v>
+      </c>
+      <c r="Q6" t="s">
+        <v>69</v>
+      </c>
+      <c r="R6" t="s">
+        <v>75</v>
+      </c>
+      <c r="S6" t="s">
+        <v>53</v>
+      </c>
+      <c r="W6">
+        <v>1</v>
+      </c>
+      <c r="X6" t="s">
+        <v>62</v>
+      </c>
+      <c r="Y6" t="s">
+        <v>51</v>
+      </c>
+      <c r="Z6" t="s">
+        <v>217</v>
+      </c>
+      <c r="AA6" t="s">
+        <v>51</v>
+      </c>
+      <c r="AB6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AC6" t="s">
+        <v>53</v>
+      </c>
+      <c r="AD6" t="s">
+        <v>64</v>
+      </c>
+      <c r="AE6" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="7" spans="1:31" x14ac:dyDescent="0.2">
+      <c r="A7">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="8" spans="1:31" x14ac:dyDescent="0.2">
+      <c r="A8">
+        <v>25</v>
+      </c>
+      <c r="B8">
+        <v>0</v>
+      </c>
+      <c r="C8" t="s">
+        <v>51</v>
+      </c>
+      <c r="D8" t="s">
+        <v>51</v>
+      </c>
+      <c r="E8" t="s">
+        <v>51</v>
+      </c>
+      <c r="F8" t="s">
+        <v>51</v>
+      </c>
+      <c r="G8" t="s">
+        <v>50</v>
+      </c>
+      <c r="H8" t="s">
+        <v>50</v>
+      </c>
+      <c r="I8" t="s">
+        <v>50</v>
+      </c>
+      <c r="J8" t="s">
+        <v>55</v>
+      </c>
+      <c r="K8" t="s">
+        <v>50</v>
+      </c>
+      <c r="L8" t="s">
+        <v>73</v>
+      </c>
+      <c r="M8" t="s">
+        <v>51</v>
+      </c>
+      <c r="N8" t="s">
+        <v>72</v>
+      </c>
+      <c r="O8" t="s">
+        <v>51</v>
+      </c>
+      <c r="P8" t="s">
+        <v>110</v>
+      </c>
+      <c r="Q8" t="s">
+        <v>51</v>
+      </c>
+      <c r="R8">
+        <v>1</v>
+      </c>
+      <c r="S8" t="s">
+        <v>51</v>
+      </c>
+      <c r="T8" t="s">
+        <v>218</v>
+      </c>
+      <c r="U8">
+        <v>1</v>
+      </c>
+      <c r="V8" t="s">
+        <v>219</v>
+      </c>
+      <c r="W8" t="s">
+        <v>51</v>
+      </c>
+      <c r="X8" t="s">
+        <v>106</v>
+      </c>
+      <c r="Y8">
+        <v>1</v>
+      </c>
+      <c r="Z8" t="s">
+        <v>60</v>
+      </c>
+      <c r="AB8" t="s">
+        <v>75</v>
+      </c>
+      <c r="AC8" t="s">
+        <v>108</v>
+      </c>
+      <c r="AD8" t="s">
+        <v>51</v>
+      </c>
+      <c r="AE8" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="9" spans="1:31" x14ac:dyDescent="0.2">
+      <c r="A9">
+        <v>33</v>
+      </c>
+      <c r="B9" t="s">
+        <v>50</v>
+      </c>
+      <c r="C9" t="s">
+        <v>50</v>
+      </c>
+      <c r="D9">
+        <v>1</v>
+      </c>
+      <c r="E9" t="s">
+        <v>54</v>
+      </c>
+      <c r="F9" t="s">
+        <v>51</v>
+      </c>
+      <c r="G9" t="s">
+        <v>51</v>
+      </c>
+      <c r="H9" t="s">
+        <v>49</v>
+      </c>
+      <c r="I9" t="s">
+        <v>55</v>
+      </c>
+      <c r="J9" t="s">
+        <v>51</v>
+      </c>
+      <c r="K9" t="s">
+        <v>51</v>
+      </c>
+      <c r="L9" t="s">
+        <v>129</v>
+      </c>
+      <c r="M9" t="s">
+        <v>51</v>
+      </c>
+      <c r="N9" t="s">
+        <v>107</v>
+      </c>
+      <c r="O9" t="s">
+        <v>51</v>
+      </c>
+      <c r="P9" t="s">
+        <v>72</v>
+      </c>
+      <c r="Q9" t="s">
+        <v>50</v>
+      </c>
+      <c r="R9" t="s">
+        <v>51</v>
+      </c>
+      <c r="S9" t="s">
+        <v>110</v>
+      </c>
+      <c r="T9">
+        <v>1</v>
+      </c>
+      <c r="U9" t="s">
+        <v>68</v>
+      </c>
+      <c r="V9" t="s">
+        <v>51</v>
+      </c>
+      <c r="W9" t="s">
+        <v>57</v>
+      </c>
+      <c r="X9" t="s">
+        <v>51</v>
+      </c>
+      <c r="Y9" t="s">
+        <v>106</v>
+      </c>
+      <c r="Z9" t="s">
+        <v>51</v>
+      </c>
+      <c r="AA9" t="s">
+        <v>51</v>
+      </c>
+      <c r="AB9" t="s">
+        <v>51</v>
+      </c>
+      <c r="AC9">
+        <v>1</v>
+      </c>
+      <c r="AD9" t="s">
+        <v>220</v>
+      </c>
+      <c r="AE9" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="10" spans="1:31" x14ac:dyDescent="0.2">
+      <c r="A10">
+        <v>35</v>
+      </c>
+      <c r="B10">
+        <v>1</v>
+      </c>
+      <c r="C10" t="s">
+        <v>60</v>
+      </c>
+      <c r="D10" t="s">
+        <v>68</v>
+      </c>
+      <c r="E10" t="s">
+        <v>49</v>
+      </c>
+      <c r="F10" t="s">
+        <v>59</v>
+      </c>
+      <c r="G10" t="s">
+        <v>68</v>
+      </c>
+      <c r="H10" t="s">
+        <v>51</v>
+      </c>
+      <c r="I10">
+        <v>1</v>
+      </c>
+      <c r="J10" t="s">
+        <v>58</v>
+      </c>
+      <c r="K10" t="s">
+        <v>59</v>
+      </c>
+      <c r="L10" t="s">
+        <v>51</v>
+      </c>
+      <c r="M10" t="s">
+        <v>109</v>
+      </c>
+      <c r="N10">
+        <v>1</v>
+      </c>
+      <c r="O10" t="s">
+        <v>55</v>
+      </c>
+      <c r="P10" t="s">
+        <v>55</v>
+      </c>
+      <c r="Q10" t="s">
+        <v>55</v>
+      </c>
+      <c r="R10" t="s">
+        <v>51</v>
+      </c>
+      <c r="S10" t="s">
+        <v>55</v>
+      </c>
+      <c r="U10" t="s">
+        <v>68</v>
+      </c>
+      <c r="V10">
+        <v>1</v>
+      </c>
+      <c r="W10" t="s">
+        <v>55</v>
+      </c>
+      <c r="X10">
+        <v>1</v>
+      </c>
+      <c r="Y10" t="s">
+        <v>129</v>
+      </c>
+      <c r="Z10">
+        <v>1</v>
+      </c>
+      <c r="AA10">
+        <v>1</v>
+      </c>
+      <c r="AB10">
+        <v>1</v>
+      </c>
+      <c r="AC10" t="s">
+        <v>77</v>
+      </c>
+      <c r="AD10">
+        <v>1</v>
+      </c>
+      <c r="AE10" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="11" spans="1:31" x14ac:dyDescent="0.2">
+      <c r="A11">
+        <v>55</v>
+      </c>
+      <c r="D11">
+        <v>1</v>
+      </c>
+      <c r="N11">
+        <v>0</v>
+      </c>
+      <c r="P11">
+        <v>0</v>
+      </c>
+      <c r="Q11">
+        <v>1</v>
+      </c>
+      <c r="T11">
+        <v>0</v>
+      </c>
+      <c r="U11">
+        <v>1</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0641AAE6-D311-C94D-A1AC-5ABF7C834903}">
+  <dimension ref="A1:U11"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetData>
+    <row r="1" spans="1:21" x14ac:dyDescent="0.2">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>117</v>
+      </c>
+      <c r="C1" t="s">
+        <v>118</v>
+      </c>
+      <c r="D1" t="s">
+        <v>193</v>
+      </c>
+      <c r="E1" t="s">
+        <v>194</v>
+      </c>
+      <c r="F1" t="s">
+        <v>195</v>
+      </c>
+      <c r="G1" t="s">
+        <v>196</v>
+      </c>
+      <c r="H1" t="s">
+        <v>197</v>
+      </c>
+      <c r="I1" t="s">
+        <v>198</v>
+      </c>
+      <c r="J1" t="s">
+        <v>199</v>
+      </c>
+      <c r="K1" t="s">
+        <v>200</v>
+      </c>
+      <c r="L1" t="s">
+        <v>201</v>
+      </c>
+      <c r="M1" t="s">
+        <v>202</v>
+      </c>
+      <c r="N1" t="s">
+        <v>203</v>
+      </c>
+      <c r="O1" t="s">
+        <v>204</v>
+      </c>
+      <c r="P1" t="s">
+        <v>205</v>
+      </c>
+      <c r="Q1" t="s">
+        <v>206</v>
+      </c>
+      <c r="R1" t="s">
+        <v>207</v>
+      </c>
+      <c r="S1" t="s">
+        <v>208</v>
+      </c>
+      <c r="T1" t="s">
+        <v>209</v>
+      </c>
+      <c r="U1" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="2" spans="1:21" x14ac:dyDescent="0.2">
+      <c r="A2">
+        <v>11</v>
+      </c>
+      <c r="B2" t="s">
+        <v>72</v>
+      </c>
+      <c r="C2" t="s">
+        <v>49</v>
+      </c>
+      <c r="D2" t="s">
+        <v>59</v>
+      </c>
+      <c r="E2" t="s">
+        <v>67</v>
+      </c>
+      <c r="F2">
+        <v>1</v>
+      </c>
+      <c r="G2" t="s">
+        <v>67</v>
+      </c>
+      <c r="H2" t="s">
+        <v>51</v>
+      </c>
+      <c r="I2" t="s">
+        <v>51</v>
+      </c>
+      <c r="J2" t="s">
+        <v>76</v>
+      </c>
+      <c r="K2">
+        <v>1</v>
+      </c>
+      <c r="N2" t="s">
+        <v>60</v>
+      </c>
+      <c r="O2">
+        <v>1</v>
+      </c>
+      <c r="P2" t="s">
+        <v>68</v>
+      </c>
+      <c r="Q2">
+        <v>0</v>
+      </c>
+      <c r="R2" t="s">
+        <v>58</v>
+      </c>
+      <c r="S2">
+        <v>1</v>
+      </c>
+      <c r="T2" t="s">
+        <v>222</v>
+      </c>
+      <c r="U2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:21" x14ac:dyDescent="0.2">
+      <c r="A3">
+        <v>12</v>
+      </c>
+      <c r="D3" t="s">
+        <v>51</v>
+      </c>
+      <c r="E3" t="s">
+        <v>60</v>
+      </c>
+      <c r="F3">
+        <v>1</v>
+      </c>
+      <c r="G3" t="s">
+        <v>51</v>
+      </c>
+      <c r="H3">
+        <v>0</v>
+      </c>
+      <c r="I3" t="s">
+        <v>55</v>
+      </c>
+      <c r="J3" t="s">
+        <v>69</v>
+      </c>
+      <c r="K3">
+        <v>0</v>
+      </c>
+      <c r="L3" t="s">
+        <v>49</v>
+      </c>
+      <c r="M3">
+        <v>1</v>
+      </c>
+      <c r="N3">
+        <v>0</v>
+      </c>
+      <c r="O3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P3" t="s">
+        <v>68</v>
+      </c>
+      <c r="Q3" t="s">
+        <v>54</v>
+      </c>
+      <c r="R3">
+        <v>1</v>
+      </c>
+      <c r="S3" t="s">
+        <v>55</v>
+      </c>
+      <c r="T3" t="s">
+        <v>51</v>
+      </c>
+      <c r="U3" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="4" spans="1:21" x14ac:dyDescent="0.2">
+      <c r="A4">
+        <v>13</v>
+      </c>
+      <c r="D4">
+        <v>1</v>
+      </c>
+      <c r="E4" t="s">
+        <v>60</v>
+      </c>
+      <c r="F4">
+        <v>1</v>
+      </c>
+      <c r="G4">
+        <v>1</v>
+      </c>
+      <c r="H4" t="s">
+        <v>72</v>
+      </c>
+      <c r="I4" t="s">
+        <v>55</v>
+      </c>
+      <c r="J4">
+        <v>1</v>
+      </c>
+      <c r="K4" t="s">
+        <v>221</v>
+      </c>
+      <c r="L4">
+        <v>1</v>
+      </c>
+      <c r="N4" t="s">
+        <v>222</v>
+      </c>
+      <c r="O4" t="s">
+        <v>51</v>
+      </c>
+      <c r="P4" t="s">
+        <v>81</v>
+      </c>
+      <c r="Q4" t="s">
+        <v>68</v>
+      </c>
+      <c r="R4">
+        <v>1</v>
+      </c>
+      <c r="S4">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" spans="1:21" x14ac:dyDescent="0.2">
+      <c r="A5">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="6" spans="1:21" x14ac:dyDescent="0.2">
+      <c r="A6">
+        <v>22</v>
+      </c>
+      <c r="B6" t="s">
+        <v>49</v>
+      </c>
+      <c r="C6" t="s">
+        <v>80</v>
+      </c>
+      <c r="D6">
+        <v>1</v>
+      </c>
+      <c r="E6" t="s">
+        <v>125</v>
+      </c>
+      <c r="F6" t="s">
+        <v>51</v>
+      </c>
+      <c r="G6" t="s">
+        <v>51</v>
+      </c>
+      <c r="H6" t="s">
+        <v>131</v>
+      </c>
+      <c r="I6" t="s">
+        <v>55</v>
+      </c>
+      <c r="J6" t="s">
+        <v>73</v>
+      </c>
+      <c r="K6" t="s">
+        <v>51</v>
+      </c>
+      <c r="L6" t="s">
+        <v>51</v>
+      </c>
+      <c r="M6" t="s">
+        <v>51</v>
+      </c>
+      <c r="N6" t="s">
+        <v>222</v>
+      </c>
+      <c r="O6" t="s">
+        <v>51</v>
+      </c>
+      <c r="P6" t="s">
+        <v>81</v>
+      </c>
+      <c r="Q6" t="s">
+        <v>68</v>
+      </c>
+      <c r="R6" t="s">
+        <v>51</v>
+      </c>
+      <c r="S6" t="s">
+        <v>127</v>
+      </c>
+      <c r="T6" t="s">
+        <v>51</v>
+      </c>
+      <c r="U6" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="7" spans="1:21" x14ac:dyDescent="0.2">
+      <c r="A7">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="8" spans="1:21" x14ac:dyDescent="0.2">
+      <c r="A8">
+        <v>25</v>
+      </c>
+      <c r="B8" t="s">
+        <v>50</v>
+      </c>
+      <c r="C8" t="s">
+        <v>51</v>
+      </c>
+      <c r="D8" t="s">
+        <v>133</v>
+      </c>
+      <c r="E8">
+        <v>1</v>
+      </c>
+      <c r="F8" t="s">
+        <v>128</v>
+      </c>
+      <c r="G8" t="s">
+        <v>81</v>
+      </c>
+      <c r="H8" t="s">
+        <v>50</v>
+      </c>
+      <c r="I8" t="s">
+        <v>51</v>
+      </c>
+      <c r="J8" t="s">
+        <v>223</v>
+      </c>
+      <c r="K8" t="s">
+        <v>51</v>
+      </c>
+      <c r="N8" t="s">
+        <v>60</v>
+      </c>
+      <c r="O8" t="s">
+        <v>51</v>
+      </c>
+      <c r="P8">
+        <v>1</v>
+      </c>
+      <c r="Q8" t="s">
+        <v>51</v>
+      </c>
+      <c r="R8" t="s">
+        <v>55</v>
+      </c>
+      <c r="S8" t="s">
+        <v>73</v>
+      </c>
+      <c r="T8" t="s">
+        <v>64</v>
+      </c>
+      <c r="U8" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="9" spans="1:21" x14ac:dyDescent="0.2">
+      <c r="A9">
+        <v>33</v>
+      </c>
+      <c r="B9">
+        <v>0</v>
+      </c>
+      <c r="C9" t="s">
+        <v>55</v>
+      </c>
+      <c r="D9" t="s">
+        <v>49</v>
+      </c>
+      <c r="E9" t="s">
+        <v>54</v>
+      </c>
+      <c r="F9" t="s">
+        <v>51</v>
+      </c>
+      <c r="G9" t="s">
+        <v>51</v>
+      </c>
+      <c r="H9">
+        <v>1</v>
+      </c>
+      <c r="I9" t="s">
+        <v>64</v>
+      </c>
+      <c r="J9" t="s">
+        <v>51</v>
+      </c>
+      <c r="K9" t="s">
+        <v>51</v>
+      </c>
+      <c r="L9">
+        <v>1</v>
+      </c>
+      <c r="M9" t="s">
+        <v>55</v>
+      </c>
+      <c r="N9" t="s">
+        <v>68</v>
+      </c>
+      <c r="O9">
+        <v>0</v>
+      </c>
+      <c r="P9">
+        <v>0</v>
+      </c>
+      <c r="Q9" t="s">
+        <v>60</v>
+      </c>
+      <c r="R9" t="s">
+        <v>51</v>
+      </c>
+      <c r="S9">
+        <v>0</v>
+      </c>
+      <c r="U9" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="10" spans="1:21" x14ac:dyDescent="0.2">
+      <c r="A10">
+        <v>35</v>
+      </c>
+      <c r="B10" t="s">
+        <v>56</v>
+      </c>
+      <c r="E10">
+        <v>1</v>
+      </c>
+      <c r="F10" t="s">
+        <v>129</v>
+      </c>
+      <c r="G10" t="s">
+        <v>67</v>
+      </c>
+      <c r="I10">
+        <v>1</v>
+      </c>
+      <c r="J10" t="s">
+        <v>72</v>
+      </c>
+      <c r="L10" t="s">
+        <v>106</v>
+      </c>
+      <c r="N10" t="s">
+        <v>51</v>
+      </c>
+      <c r="O10">
+        <v>0</v>
+      </c>
+      <c r="P10">
+        <v>1</v>
+      </c>
+      <c r="Q10">
+        <v>1</v>
+      </c>
+      <c r="R10" t="s">
+        <v>127</v>
+      </c>
+      <c r="S10">
+        <v>1</v>
+      </c>
+      <c r="T10" t="s">
+        <v>132</v>
+      </c>
+      <c r="U10">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="11" spans="1:21" x14ac:dyDescent="0.2">
+      <c r="A11">
+        <v>55</v>
+      </c>
+      <c r="D11">
+        <v>1</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>